<commit_message>
added some test data #23
</commit_message>
<xml_diff>
--- a/data/world_data.xlsx
+++ b/data/world_data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\simon\Downloads\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Skole\uni\Bachelor\Bachelor-Projekt\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B9332717-FB7D-4561-A494-24D6E09033EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{272CBE9B-B16C-4C32-9977-C1155192C830}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" xr2:uid="{C1B2DA82-B258-4471-8CF0-4CEB24F6CDE7}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="54">
   <si>
     <t>quests</t>
   </si>
@@ -6807,6 +6807,58 @@
   "Skills": [{"Name": "One-Handed", "Level": 25}, {"Name": "Lockpicking", "Level": 15}]
 }
 ;</t>
+  </si>
+  <si>
+    <t>testdata</t>
+  </si>
+  <si>
+    <t>## ENUM DATA
+//enum data here
+;
+## GAME STATE DATA
+### NPC DATA
+Thalia Ironvein: {"Name":"Thalia Ironvein","Species":"Dwarf","HomeLocation":"Ironhold Keep","CurrentLocation":"Ironhold Keep","Faction":"Miners Guild","OwnedItems":{"Iron Ore":5,"Pickaxe":1},"Role":"Foreman","Relations":[{"Target":"Player","Favorability":"Ally"}],"NPCLog":[]}
+;
+Eldrin Moonshadow: {"Name":"Eldrin Moonshadow","Species":"Elf","HomeLocation":"Silverwood Grove","CurrentLocation":"Whispering Ruins","Faction":"Wildborne Circle","OwnedItems":{"Healing Herb":3,"Ancient Scroll":1},"Role":"Scout","Relations":[{"Target":"Player","Favorability":"Neutral"},{"Target":"Miners Guild","Favorability":"Enemy"}],"NPCLog":[]}
+;
+Gromm Stonefist: {"Name":"Gromm Stonefist","Species":"Orc","HomeLocation":"Bloodhoof Village","CurrentLocation":"Bloodhoof Village","Faction":"Iron Horde","OwnedItems":{"War Axe":1,"Meat":2},"Role":"Warrior","Relations":[{"Target":"Player","Favorability":"Sworn Enemy"}],"NPCLog":[]}
+;
+Seraphina Dawn: {"Name":"Seraphina Dawn","Species":"Human","HomeLocation":"Havenport","CurrentLocation":"Havenport","Faction":"Crimson Dawn","OwnedItems":{"Holy Symbol":1,"Potion":2},"Role":"Healer","Relations":[{"Target":"Player","Favorability":"Sworn Ally"}],"NPCLog":[]}
+;
+Kaelen Windstrider: {"Name":"Kaelen Windstrider","Species":"Elf","HomeLocation":"Silverwood Grove","CurrentLocation":"Havenport","Faction":"Wildborne Circle","OwnedItems":{"Bow":1,"Arrow":20},"Role":"Ranger","Relations":[{"Target":"Player","Favorability":"Ally"}],"NPCLog":[]}
+;
+Mira Swiftfoot: {"Name":"Mira Swiftfoot","Species":"Halfling","HomeLocation":"Havenport","CurrentLocation":"Havenport","Faction":"Thieves Guild","OwnedItems":{"Lockpick":5,"Gold":50},"Role":"Rogue","Relations":[{"Target":"Player","Favorability":"Friendly"}],"NPCLog":[]}
+;
+Borak Ironhide: {"Name":"Borak Ironhide","Species":"Orc","HomeLocation":"Bloodhoof Village","CurrentLocation":"Ironhold Keep","Faction":"Miners Guild","OwnedItems":{"Mining Helmet":1,"Dynamite":2},"Role":"Laborer","Relations":[{"Target":"Player","Favorability":"Neutral"}],"NPCLog":[]}
+;
+Lyra Emberheart: {"Name":"Lyra Emberheart","Species":"Human","HomeLocation":"Havenport","CurrentLocation":"Cinderfall Mine","Faction":"Crimson Dawn","OwnedItems":{"Fire Staff":1,"Fire Gem":1},"Role":"Mage","Relations":[{"Target":"Player","Favorability":"Ally"}],"NPCLog":[]}
+;
+Rurik Shattershield: {"Name":"Rurik Shattershield","Species":"Dwarf","HomeLocation":"Ironhold Keep","CurrentLocation":"Ironhold Keep","Faction":"Iron Horde","OwnedItems":{"Shield":1,"Axe":1},"Role":"Captain","Relations":[{"Target":"Player","Favorability":"Enemy"}],"NPCLog":[]}
+;
+Vex Shadowtongue: {"Name":"Vex Shadowtongue","Species":"Halfling","HomeLocation":"Havenport","CurrentLocation":"Whispering Ruins","Faction":"Thieves Guild","OwnedItems":{"Poison":3,"Throwing Knife":4},"Role":"Assassin","Relations":[{"Target":"Player","Favorability":"Sworn Enemy"}],"NPCLog":[]}
+;
+### FACTION DATA
+Miners Guild: {"Name":"Miners Guild","Relations":[{"Target":"Wildborne Circle","Favorability":"Ally"},{"Target":"Iron Horde","Favorability":"Enemy"},{"Target":"Player","Favorability":"Friendly"}],"Members":["Thalia Ironvein","Borak Ironhide"],"Treasury":{"Gold":500,"Iron Ore":200},"FactionLog":[]}
+;
+Wildborne Circle: {"Name":"Wildborne Circle","Relations":[{"Target":"Miners Guild","Favorability":"Ally"},{"Target":"Crimson Dawn","Favorability":"Neutral"},{"Target":"Player","Favorability":"Sworn Ally"}],"Members":["Eldrin Moonshadow","Kaelen Windstrider"],"Treasury":{"Healing Herb":50,"Ancient Wood":30},"FactionLog":[]}
+;
+Iron Horde: {"Name":"Iron Horde","Relations":[{"Target":"Miners Guild","Favorability":"Sworn Enemy"},{"Target":"Crimson Dawn","Favorability":"Enemy"},{"Target":"Player","Favorability":"Sworn Enemy"}],"Members":["Gromm Stonefist","Rurik Shattershield"],"Treasury":{"War Axe":10,"Gold":300},"FactionLog":[]}
+;
+### ENEMY DATA
+Cave Troll: {"Name":"Cave Troll","Loot":["Troll Hide","Gold","Troll Bone"]}
+;
+Shadow Wraith: {"Name":"Shadow Wraith","Loot":["Ectoplasm","Shadow Essence"]}
+;
+Iron Horde Marauder: {"Name":"Iron Horde Marauder","Loot":["Iron Sword","Gold","Health Potion"]}
+;
+Cinder Elemental: {"Name":"Cinder Elemental","Loot":["Fire Crystal","Ash Powder"]}
+;
+Forest Spider: {"Name":"Forest Spider","Loot":["Spider Silk","Venom Gland"]}
+;
+;## PLAYER DATA
+{"Species":"Human","FactionRelations":[{"Target":"Miners Guild","Favorability":"Friendly"},{"Target":"Wildborne Circle","Favorability":"Sworn Ally"},{"Target":"Iron Horde","Favorability":"Sworn Enemy"}],"NPCRelations":[{"Target":"Thalia Ironvein","Favorability":"Ally"},{"Target":"Eldrin Moonshadow","Favorability":"Neutral"},{"Target":"Gromm Stonefist","Favorability":"Sworn Enemy"},{"Target":"Seraphina Dawn","Favorability":"Sworn Ally"},{"Target":"Kaelen Windstrider","Favorability":"Ally"},{"Target":"Mira Swiftfoot","Favorability":"Friendly"},{"Target":"Borak Ironhide","Favorability":"Neutral"},{"Target":"Lyra Emberheart","Favorability":"Ally"},{"Target":"Rurik Shattershield","Favorability":"Enemy"},{"Target":"Vex Shadowtongue","Favorability":"Sworn Enemy"}],"PartyMembers":["Seraphina Dawn","Kaelen Windstrider","Mira Swiftfoot"],"Inventory":{"Iron Sword":1,"Health Potion":5,"Gold":250,"Healing Herb":10,"Lockpick":3},"PlayerLog":[{"Originator":"Player","Type":"KillEnemies","Target":["Cave Troll"],"For":"Player","Received":{"Gold":50,"Troll Hide":1},"Favorability":5},{"Originator":"Player","Type":"RecoverStolenItem","Target":["Ancient Scroll"],"For":"Wildborne Circle","Received":{"FactionReputation":15},"Favorability":10},{"Originator":"Wildborne Circle","Type":"QuestTypes","Target":["Cinder Elemental"],"For":"Player","Received":{"Gold":80},"Favorability":8},{"Originator":"Player","Type":"KillEnemies","Target":["Iron Horde Marauder"],"For":"Miners Guild","Received":{"Gold":30},"Favorability":4},{"Originator":"Miners Guild","Type":"QuestTypes","Target":["Iron Horde"],"For":"Player","Received":{"Iron Ore":15},"Favorability":6},{"Originator":"Player","Type":"GuardEntity","Target":["Seraphina Dawn"],"For":"Crimson Dawn","Received":{"Potion":2},"Favorability":7},{"Originator":"Iron Horde","Type":"AttackEnemy","Target":["Player"],"For":"Iron Horde","Received":null,"Favorability":-5},{"Originator":"Player","Type":"StealStuff","Target":["Iron Horde Treasury"],"For":"Player","Received":{"Gold":100,"War Axe":1},"Favorability":-8},{"Originator":"Player","Type":"KillEnemies","Target":["Shadow Wraith"],"For":"Wildborne Circle","Received":{"Shadow Essence":1},"Favorability":9},{"Originator":"Thieves Guild","Type":"QuestTypes","Target":["Rurik Shattershield"],"For":"Player","Received":{"Gold":60},"Favorability":6}],"Location":"Havenport","Skills":[{"Name":"Swordsmanship","Level":4},{"Name":"Stealth","Level":3},{"Name":"Persuasion","Level":2}]}
+;
+## Content</t>
   </si>
 </sst>
 </file>
@@ -7189,29 +7241,39 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16B9A6FD-C15A-4AE9-97D7-752FDF6346C0}">
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="24.21875" customWidth="1"/>
+    <col min="8" max="8" width="18.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
+      <c r="H1" t="s">
+        <v>1</v>
+      </c>
     </row>
-    <row r="2" spans="1:2" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>27</v>
       </c>
+      <c r="G2" t="s">
+        <v>52</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>53</v>
+      </c>
     </row>
-    <row r="3" spans="1:2" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
@@ -7219,7 +7281,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -7227,7 +7289,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>2</v>
       </c>
@@ -7235,7 +7297,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
@@ -7243,7 +7305,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="12.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="12.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>7</v>
       </c>
@@ -7251,7 +7313,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>8</v>
       </c>
@@ -7259,7 +7321,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>9</v>
       </c>
@@ -7267,7 +7329,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>10</v>
       </c>
@@ -7275,7 +7337,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="12.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="12.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>11</v>
       </c>
@@ -7283,7 +7345,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>12</v>
       </c>
@@ -7291,7 +7353,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>13</v>
       </c>
@@ -7299,7 +7361,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>14</v>
       </c>
@@ -7307,7 +7369,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>15</v>
       </c>
@@ -7315,7 +7377,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>16</v>
       </c>

</xml_diff>

<commit_message>
#23 more data and updates to llm inputs
</commit_message>
<xml_diff>
--- a/data/world_data.xlsx
+++ b/data/world_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Skole\uni\Bachelor\Bachelor-Projekt\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9B8F4FB-A60A-4D3F-841E-C64C3CD5C1CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{511AF175-BAAC-47A7-8722-63625D1AE376}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" xr2:uid="{C1B2DA82-B258-4471-8CF0-4CEB24F6CDE7}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="45">
   <si>
     <t>quests</t>
   </si>
@@ -16183,1014 +16183,6 @@
 Luc</t>
   </si>
   <si>
-    <t>## ENUM DATA
-{
-  "Types": {
-    "ItemTypes": ["Weapon", "Armor", "Potion", "Ingredient", "Key", "Artifact", "Currency", "Shield", "Scroll", "Food"],
-    "QuestTypes": ["AttackThreateningEntities", "RecoverStolenItem", "GuardEntity", "AttackEnemy", "StealStuff", "KillEnemies"],
-    "EventTypes": ["Ambush", "Discovery", "Betrayal", "Alliance", "TradeRouteOpened", "ResourceDepleted", "Theft", "Rescue", "CraftingSuccess", "FactionShift"],
-    "RelationshipLevels": {"Sworn Enemy" : -50, "Enemy" : -30, "Hated" : -15, "Disliked" : -5, "Neutral" : 0, "Friendly" : 5, "Friend" : 15, "Ally" : 30, "Sworn Ally" : 50}
-  },
-  "Lists": {
-    "Species": ["Human", "Elf", "Dwarf", "Orc", "Halfling", "Lizardfolk", "Half-Elf", "Goblin", "Troll", "Skeleton"],
-    "Roles": ["Innkeeper", "Blacksmith", "Merchant", "GuardCaptain", "Apothecary", "Thief", "Wizard", "Ranger", "Bard", "Priest", "Alchemist", "Farmer", "Mercenary", "Spy", "Noble", "Beggar", "Hunter", "Fisherman", "Tailor", "Jeweler"],
-    "Locations": ["Verdantia", "Ironhold", "Whispering Woods", "Crimson Badlands", "Silverport", "Elderforge Mountain", "The Sinking Marshes", "Sunstone Oasis", "Frostveil Tundra", "Shadowfen Swamp"],
-    "Factions": ["The Iron Circle", "Verdant Enclave", "Crimson Marauders", "The Silent Coin", "The Keepers of the Forge"],
-    "Enemies": ["Forest Spider", "Swamp Ghoul", "Bandit Archer", "Cave Troll", "Skeleton Warrior", "Mudcrab", "Dire Wolf", "Harpy", "Goblin Scavenger", "Orc Berserker", "Shadow Wraith", "Rock Elemental", "Venomous Bat", "Frost Spider", "Desert Scorpion", "Pirate Raider", "Cultist Acolyte", "Rogue Automaton", "Mountain Bear", "Slime Ooze"],
-    "Items": ["Iron Longsword", "Elven Shortbow", "Steel Dagger", "Health Potion", "Mana Vial", "Stamina Drought", "Nightshade Petal", "Glowdust", "Ancient Grimoire", "Merchant's Ledger", "Silver Key", "Golden Chalice", "Enchanted Amulet", "Obsidian Shard", "Copper Coin", "Silver Mark", "Gold Crown", "Iron Shield", "Leather Armor", "Chainmail Vest", "Mage Robe", "Traveling Cloak", "Lockpicks", "Bear Trap", "Smoke Bomb", "Cooking Spices", "Salted Meat", "Fresh Water", "Dwarven Ale", "Elven Bread"],
-    "NPCs": ["Elderon Greenscale", "Kaelen Swiftarrow", "Durin Stonebrow", "Lyra Silvertongue", "Grimmok Bloodfist", "Pippin Thistlefoot", "Seraphina Dawnseeker", "Borin Ironfoot", "Sasha Voss", "Marcus Reed", "Isolde", "Thrain Coalbeard", "Elara Moonshadow", "Roric", "Gretta", "Jasper Finn", "Nyx", "Captain Valeria Holt", "Barnaby Cole", "Whispering Willow", "Zargoth the Melodious", "Father Dominic", "Helga Giantbone", "Finnian", "Click-Clack", "Boulder", "Morgan Ashford", "Silas Darkwater", "Veronica Vane", "Chief Urgnak", "Talia Ironvein", "Roderick", "Squeak", "Madame Zephyra", "Corvus", "Garrick", "Mira", "Drogan", "Lysander", "Pearl", "Rusty Rivet", "Bram Heston", "Opal", "Grizzle Geargrinder", "Vanya", "Flick", "Yorick", "Anya", "Cyrus the Cursed", "Roland the Stout"],
-    "Player": ["The Traveler"]
-  }
-}
-;
-### ITEM DATA
-Iron Longsword: { 
-  "Type": "Weapon", 
-  "Name": "Iron Longsword", 
-  "NameSingular": "iron longsword", 
-  "NamePlural": "iron longswords",
-  "NamePossessiveSingular": "iron longsword's",
-  "NamePossessivePlural": "iron longswords'",
-  "IndefiniteArticle": "an",
-  "IndefiniteArticleCaps": "An"
-}
-Elven Shortbow: { 
-  "Type": "Weapon", 
-  "Name": "Elven Shortbow", 
-  "NameSingular": "elven shortbow", 
-  "NamePlural": "elven shortbows",
-  "NamePossessiveSingular": "elven shortbow's",
-  "NamePossessivePlural": "elven shortbows'",
-  "IndefiniteArticle": "an",
-  "IndefiniteArticleCaps": "An"
-}
-Steel Dagger: { 
-  "Type": "Weapon", 
-  "Name": "Steel Dagger", 
-  "NameSingular": "steel dagger", 
-  "NamePlural": "steel daggers",
-  "NamePossessiveSingular": "steel dagger's",
-  "NamePossessivePlural": "steel daggers'",
-  "IndefiniteArticle": "a",
-  "IndefiniteArticleCaps": "A"
-}
-Health Potion: { 
-  "Type": "Potion", 
-  "Name": "Health Potion", 
-  "NameSingular": "health potion", 
-  "NamePlural": "health potions",
-  "NamePossessiveSingular": "health potion's",
-  "NamePossessivePlural": "health potions'",
-  "IndefiniteArticle": "a",
-  "IndefiniteArticleCaps": "A"
-}
-Mana Vial: { 
-  "Type": "Potion", 
-  "Name": "Mana Vial", 
-  "NameSingular": "mana vial", 
-  "NamePlural": "mana vials",
-  "NamePossessiveSingular": "mana vial's",
-  "NamePossessivePlural": "mana vials'",
-  "IndefiniteArticle": "a",
-  "IndefiniteArticleCaps": "A"
-}
-Stamina Drought: { 
-  "Type": "Potion", 
-  "Name": "Stamina Drought", 
-  "NameSingular": "stamina drought", 
-  "NamePlural": "stamina droughts",
-  "NamePossessiveSingular": "stamina drought's",
-  "NamePossessivePlural": "stamina droughts'",
-  "IndefiniteArticle": "a",
-  "IndefiniteArticleCaps": "A"
-}
-Nightshade Petal: { 
-  "Type": "Ingredient", 
-  "Name": "Nightshade Petal", 
-  "NameSingular": "nightshade petal", 
-  "NamePlural": "nightshade petals",
-  "NamePossessiveSingular": "nightshade petal's",
-  "NamePossessivePlural": "nightshade petals'",
-  "IndefiniteArticle": "a",
-  "IndefiniteArticleCaps": "A"
-}
-Glowdust: { 
-  "Type": "Ingredient", 
-  "Name": "Glowdust", 
-  "NameSingular": "glowdust", 
-  "NamePlural": "glowdust",
-  "NamePossessiveSingular": "glowdust's",
-  "NamePossessivePlural": "glowdust's",
-  "IndefiniteArticle": "a",
-  "IndefiniteArticleCaps": "A"
-}
-Ancient Grimoire: { 
-  "Type": "Artifact", 
-  "Name": "Ancient Grimoire", 
-  "NameSingular": "ancient grimoire", 
-  "NamePlural": "ancient grimoires",
-  "NamePossessiveSingular": "ancient grimoire's",
-  "NamePossessivePlural": "ancient grimoires'",
-  "IndefiniteArticle": "an",
-  "IndefiniteArticleCaps": "An"
-}
-Merchant's Ledger: { 
-  "Type": "Artifact", 
-  "Name": "Merchant's Ledger", 
-  "NameSingular": "merchant's ledger", 
-  "NamePlural": "merchant's ledgers",
-  "NamePossessiveSingular": "merchant's ledger's",
-  "NamePossessivePlural": "merchant's ledgers'",
-  "IndefiniteArticle": "a",
-  "IndefiniteArticleCaps": "A"
-}
-Silver Key: { 
-  "Type": "Key", 
-  "Name": "Silver Key", 
-  "NameSingular": "silver key", 
-  "NamePlural": "silver keys",
-  "NamePossessiveSingular": "silver key's",
-  "NamePossessivePlural": "silver keys'",
-  "IndefiniteArticle": "a",
-  "IndefiniteArticleCaps": "A"
-}
-Golden Chalice: { 
-  "Type": "Artifact", 
-  "Name": "Golden Chalice", 
-  "NameSingular": "golden chalice", 
-  "NamePlural": "golden chalices",
-  "NamePossessiveSingular": "golden chalice's",
-  "NamePossessivePlural": "golden chalices'",
-  "IndefiniteArticle": "a",
-  "IndefiniteArticleCaps": "A"
-}
-Enchanted Amulet: { 
-  "Type": "Artifact", 
-  "Name": "Enchanted Amulet", 
-  "NameSingular": "enchanted amulet", 
-  "NamePlural": "enchanted amulets",
-  "NamePossessiveSingular": "enchanted amulet's",
-  "NamePossessivePlural": "enchanted amulets'",
-  "IndefiniteArticle": "an",
-  "IndefiniteArticleCaps": "An"
-}
-Obsidian Shard: { 
-  "Type": "Ingredient", 
-  "Name": "Obsidian Shard", 
-  "NameSingular": "obsidian shard", 
-  "NamePlural": "obsidian shards",
-  "NamePossessiveSingular": "obsidian shard's",
-  "NamePossessivePlural": "obsidian shards'",
-  "IndefiniteArticle": "an",
-  "IndefiniteArticleCaps": "An"
-}
-Copper Coin: { 
-  "Type": "Currency", 
-  "Name": "Copper Coin", 
-  "NameSingular": "copper coin", 
-  "NamePlural": "copper coins",
-  "NamePossessiveSingular": "copper coin's",
-  "NamePossessivePlural": "copper coins'",
-  "IndefiniteArticle": "a",
-  "IndefiniteArticleCaps": "A"
-}
-Silver Mark: { 
-  "Type": "Currency", 
-  "Name": "Silver Mark", 
-  "NameSingular": "silver mark", 
-  "NamePlural": "silver marks",
-  "NamePossessiveSingular": "silver mark's",
-  "NamePossessivePlural": "silver marks'",
-  "IndefiniteArticle": "a",
-  "IndefiniteArticleCaps": "A"
-}
-Gold Crown: { 
-  "Type": "Currency", 
-  "Name": "Gold Crown", 
-  "NameSingular": "gold crown", 
-  "NamePlural": "gold crowns",
-  "NamePossessiveSingular": "gold crown's",
-  "NamePossessivePlural": "gold crowns'",
-  "IndefiniteArticle": "a",
-  "IndefiniteArticleCaps": "A"
-}
-Iron Shield: { 
-  "Type": "Shield", 
-  "Name": "Iron Shield", 
-  "NameSingular": "iron shield", 
-  "NamePlural": "iron shields",
-  "NamePossessiveSingular": "iron shield's",
-  "NamePossessivePlural": "iron shields'",
-  "IndefiniteArticle": "an",
-  "IndefiniteArticleCaps": "An"
-}
-Leather Armor: { 
-  "Type": "Armor", 
-  "Name": "Leather Armor", 
-  "NameSingular": "leather armor", 
-  "NamePlural": "leather armors",
-  "NamePossessiveSingular": "leather armor's",
-  "NamePossessivePlural": "leather armors'",
-  "IndefiniteArticle": "a",
-  "IndefiniteArticleCaps": "A"
-}
-Chainmail Vest: { 
-  "Type": "Armor", 
-  "Name": "Chainmail Vest", 
-  "NameSingular": "chainmail vest", 
-  "NamePlural": "chainmail vests",
-  "NamePossessiveSingular": "chainmail vest's",
-  "NamePossessivePlural": "chainmail vests'",
-  "IndefiniteArticle": "a",
-  "IndefiniteArticleCaps": "A"
-}
-Mage Robe: { 
-  "Type": "Armor", 
-  "Name": "Mage Robe", 
-  "NameSingular": "mage robe", 
-  "NamePlural": "mage robes",
-  "NamePossessiveSingular": "mage robe's",
-  "NamePossessivePlural": "mage robes'",
-  "IndefiniteArticle": "a",
-  "IndefiniteArticleCaps": "A"
-}
-Traveling Cloak: { 
-  "Type": "Armor", 
-  "Name": "Traveling Cloak", 
-  "NameSingular": "traveling cloak", 
-  "NamePlural": "traveling cloaks",
-  "NamePossessiveSingular": "traveling cloak's",
-  "NamePossessivePlural": "traveling cloaks'",
-  "IndefiniteArticle": "a",
-  "IndefiniteArticleCaps": "A"
-}
-Lockpicks: { 
-  "Type": "Artifact", 
-  "Name": "Lockpicks", 
-  "NameSingular": "lockpicks", 
-  "NamePlural": "lockpicks",
-  "NamePossessiveSingular": "lockpicks'",
-  "NamePossessivePlural": "lockpicks'",
-  "IndefiniteArticle": "a set of",
-  "IndefiniteArticleCaps": "A set of"
-}
-Bear Trap: { 
-  "Type": "Artifact", 
-  "Name": "Bear Trap", 
-  "NameSingular": "bear trap", 
-  "NamePlural": "bear traps",
-  "NamePossessiveSingular": "bear trap's",
-  "NamePossessivePlural": "bear traps'",
-  "IndefiniteArticle": "a",
-  "IndefiniteArticleCaps": "A"
-}
-Smoke Bomb: { 
-  "Type": "Artifact", 
-  "Name": "Smoke Bomb", 
-  "NameSingular": "smoke bomb", 
-  "NamePlural": "smoke bombs",
-  "NamePossessiveSingular": "smoke bomb's",
-  "NamePossessivePlural": "smoke bombs'",
-  "IndefiniteArticle": "a",
-  "IndefiniteArticleCaps": "A"
-}
-Cooking Spices: { 
-  "Type": "Ingredient", 
-  "Name": "Cooking Spices", 
-  "NameSingular": "cooking spices", 
-  "NamePlural": "cooking spices",
-  "NamePossessiveSingular": "cooking spices'",
-  "NamePossessivePlural": "cooking spices'",
-  "IndefiniteArticle": "a jar of",
-  "IndefiniteArticleCaps": "A jar of"
-}
-Salted Meat: { 
-  "Type": "Food", 
-  "Name": "Salted Meat", 
-  "NameSingular": "salted meat", 
-  "NamePlural": "salted meats",
-  "NamePossessiveSingular": "salted meat's",
-  "NamePossessivePlural": "salted meats'",
-  "IndefiniteArticle": "a piece of",
-  "IndefiniteArticleCaps": "A piece of"
-}
-Fresh Water: { 
-  "Type": "Food", 
-  "Name": "Fresh Water", 
-  "NameSingular": "fresh water", 
-  "NamePlural": "fresh waters",
-  "NamePossessiveSingular": "fresh water's",
-  "NamePossessivePlural": "fresh waters'",
-  "IndefiniteArticle": "a flask of",
-  "IndefiniteArticleCaps": "A flask of"
-}
-Dwarven Ale: { 
-  "Type": "Food", 
-  "Name": "Dwarven Ale", 
-  "NameSingular": "dwarven ale", 
-  "NamePlural": "dwarven ales",
-  "NamePossessiveSingular": "dwarven ale's",
-  "NamePossessivePlural": "dwarven ales'",
-  "IndefiniteArticle": "a mug of",
-  "IndefiniteArticleCaps": "A mug of"
-}
-Elven Bread: { 
-  "Type": "Food", 
-  "Name": "Elven Bread", 
-  "NameSingular": "elven bread", 
-  "NamePlural": "elven breads",
-  "NamePossessiveSingular": "elven bread's",
-  "NamePossessivePlural": "elven breads'",
-  "IndefiniteArticle": "a loaf of",
-  "IndefiniteArticleCaps": "A loaf of"
-}
-;
-## GAME STATE DATA
-### FACTION DATA
-The Iron Circle: {
-  "Name": "The Iron Circle", 
-  "NameDefinitive": "the Iron Circle",
-  "NameDefinitiveCaps": "The Iron Circle",
-  "NamePossessive": "The Iron Circle's",
-  "NameDefinitivePossessive": "the Iron Circle's",
-  "NameDefinitivePossessiveCaps": "The Iron Circle's",
-  "DefaultLocation": "Ironhold",
-  "Relations": [
-    {"Target": "The Traveler", "Favorability": 15},
-    {"Target": "Verdant Enclave", "Favorability": -5},
-    {"Target": "Crimson Marauders", "Favorability": -30},
-    {"Target": "The Silent Coin", "Favorability": 5},
-    {"Target": "The Keepers of the Forge", "Favorability": 30}
-  ],
-  "Members": ["Captain Valeria Holt", "Marcus Reed", "Sasha Voss", "Bram Heston", "Roland the Stout"],
-  "Treasury": {
-    "Iron Longsword": 10,
-    "Iron Shield": 8,
-    "Chainmail Vest": 5,
-    "Gold Crown": 500,
-    "Salted Meat": 20
-  },
-  "FactionLog": []
-}
-Verdant Enclave: {
-  "Name": "Verdant Enclave", 
-  "NameDefinitive": "the Verdant Enclave",
-  "NameDefinitiveCaps": "The Verdant Enclave",
-  "NamePossessive": "Verdant Enclave's",
-  "NameDefinitivePossessive": "the Verdant Enclave's",
-  "NameDefinitivePossessiveCaps": "The Verdant Enclave's",
-  "DefaultLocation": "Whispering Woods",
-  "Relations": [
-    {"Target": "The Traveler", "Favorability": 30},
-    {"Target": "The Iron Circle", "Favorability": -5},
-    {"Target": "Crimson Marauders", "Favorability": -50},
-    {"Target": "The Silent Coin", "Favorability": 0},
-    {"Target": "The Keepers of the Forge", "Favorability": 15}
-  ],
-  "Members": ["Elderon Greenscale", "Kaelen Swiftarrow", "Elara Moonshadow", "Whispering Willow", "Lysander"],
-  "Treasury": {
-    "Elven Shortbow": 7,
-    "Health Potion": 15,
-    "Mana Vial": 20,
-    "Elven Bread": 30,
-    "Glowdust": 50
-  },
-  "FactionLog": []
-}
-Crimson Marauders: {
-  "Name": "Crimson Marauders", 
-  "NameDefinitive": "the Crimson Marauders",
-  "NameDefinitiveCaps": "The Crimson Marauders",
-  "NamePossessive": "Crimson Marauders'",
-  "NameDefinitivePossessive": "the Crimson Marauders'",
-  "NameDefinitivePossessiveCaps": "The Crimson Marauders'",
-  "DefaultLocation": "Crimson Badlands",
-  "Relations": [
-    {"Target": "The Traveler", "Favorability": -15},
-    {"Target": "The Iron Circle", "Favorability": -30},
-    {"Target": "Verdant Enclave", "Favorability": -50},
-    {"Target": "The Silent Coin", "Favorability": 5},
-    {"Target": "The Keepers of the Forge", "Favorability": -5}
-  ],
-  "Members": ["Grimmok Bloodfist", "Chief Urgnak", "Garrick", "Mira", "Drogan"],
-  "Treasury": {
-    "Steel Dagger": 12,
-    "Lockpicks": 4,
-    "Gold Crown": 1200,
-    "Smoke Bomb": 10,
-    "Bear Trap": 5
-  },
-  "FactionLog": []
-}
-The Silent Coin: {
-  "Name": "The Silent Coin", 
-  "NameDefinitive": "the Silent Coin",
-  "NameDefinitiveCaps": "The Silent Coin",
-  "NamePossessive": "The Silent Coin's",
-  "NameDefinitivePossessive": "the Silent Coin's",
-  "NameDefinitivePossessiveCaps": "The Silent Coin's",
-  "DefaultLocation": "Silverport",
-  "Relations": [
-    {"Target": "The Traveler", "Favorability": -5},
-    {"Target": "The Iron Circle", "Favorability": 5},
-    {"Target": "Verdant Enclave", "Favorability": 0},
-    {"Target": "Crimson Marauders", "Favorability": 5},
-    {"Target": "The Keepers of the Forge", "Favorability": 15}
-  ],
-  "Members": ["Lyra Silvertongue", "Jasper Finn", "Nyx", "Silas Darkwater", "Veronica Vane", "Flick"],
-  "Treasury": {
-    "Gold Crown": 5000,
-    "Silver Key": 3,
-    "Merchant's Ledger": 2,
-    "Traveling Cloak": 4,
-    "Lockpicks": 6
-  },
-  "FactionLog": []
-}
-The Keepers of the Forge: {
-  "Name": "The Keepers of the Forge", 
-  "NameDefinitive": "the Keepers of the Forge",
-  "NameDefinitiveCaps": "The Keepers of the Forge",
-  "NamePossessive": "The Keepers of the Forge's",
-  "NameDefinitivePossessive": "the Keepers of the Forge's",
-  "NameDefinitivePossessiveCaps": "The Keepers of the Forge's",
-  "DefaultLocation": "Elderforge Mountain",
-  "Relations": [
-    {"Target": "The Traveler", "Favorability": 15},
-    {"Target": "The Iron Circle", "Favorability": 30},
-    {"Target": "Verdant Enclave", "Favorability": 15},
-    {"Target": "Crimson Marauders", "Favorability": -5},
-    {"Target": "The Silent Coin", "Favorability": 15}
-  ],
-  "Members": ["Durin Stonebrow", "Borin Ironfoot", "Thrain Coalbeard", "Talia Ironvein", "Grizzle Geargrinder"],
-  "Treasury": {
-    "Obsidian Shard": 20,
-    "Iron Longsword": 4,
-    "Iron Shield": 4,
-    "Dwarven Ale": 25,
-    "Gold Crown": 800
-  },
-  "FactionLog": []
-}
-;
-### NPC DATA
-Elderon Greenscale: {
-  "Name": "Elderon Greenscale",
-  "NamePossessive": "Elderon Greenscale's",
-  "Species": "Lizardfolk",
-  "HomeLocation": "Whispering Woods",
-  "CurrentLocation": "Whispering Woods",
-  "Faction": "Verdant Enclave",
-  "OwnedItems": {
-    "Health Potion": 2,
-    "Ancient Grimoire": 1
-  },
-  "Role": "Wizard",
-  "Relations": [
-    {"Target": "The Traveler", "Favorability": 30},
-    {"Target": "Verdant Enclave", "Favorability": 50},
-    {"Target": "Crimson Marauders", "Favorability": -50},
-    {"Target": "Kaelen Swiftarrow", "Favorability": 30},
-    {"Target": "Elara Moonshadow", "Favorability": 35},
-    {"Target": "Whispering Willow", "Favorability": 20},
-    {"Target": "Lyra Silvertongue", "Favorability": 5},
-    {"Target": "Grimmok Bloodfist", "Favorability": -40}
-  ],
-  "NPCLog": []
-}
-Kaelen Swiftarrow: {
-  "Name": "Kaelen Swiftarrow",
-  "NamePossessive": "Kaelen Swiftarrow's",
-  "Species": "Elf",
-  "HomeLocation": "Whispering Woods",
-  "CurrentLocation": "Whispering Woods",
-  "Faction": "Verdant Enclave",
-  "OwnedItems": {
-    "Elven Shortbow": 1,
-    "Leather Armor": 1
-  },
-  "Role": "Ranger",
-  "Relations": [
-    {"Target": "The Traveler", "Favorability": 35},
-    {"Target": "Verdant Enclave", "Favorability": 45},
-    {"Target": "Crimson Marauders", "Favorability": -45},
-    {"Target": "Elderon Greenscale", "Favorability": 30},
-    {"Target": "Elara Moonshadow", "Favorability": 40},
-    {"Target": "Durin Stonebrow", "Favorability": 15},
-    {"Target": "Chief Urgnak", "Favorability": -50}
-  ],
-  "NPCLog": []
-}
-Durin Stonebrow: {
-  "Name": "Durin Stonebrow",
-  "NamePossessive": "Durin Stonebrow's",
-  "Species": "Dwarf",
-  "HomeLocation": "Elderforge Mountain",
-  "CurrentLocation": "Ironhold",
-  "Faction": "The Keepers of the Forge",
-  "OwnedItems": {
-    "Dwarven Ale": 3,
-    "Obsidian Shard": 5
-  },
-  "Role": "Blacksmith",
-  "Relations": [
-    {"Target": "The Traveler", "Favorability": 20},
-    {"Target": "The Keepers of the Forge", "Favorability": 40},
-    {"Target": "Crimson Marauders", "Favorability": -10},
-    {"Target": "Borin Ironfoot", "Favorability": 30},
-    {"Target": "Thrain Coalbeard", "Favorability": 35},
-    {"Target": "Captain Valeria Holt", "Favorability": 25},
-    {"Target": "Lyra Silvertongue", "Favorability": -5},
-    {"Target": "Sasha Voss", "Favorability": 15}
-  ],
-  "NPCLog": []
-}
-Lyra Silvertongue: {
-  "Name": "Lyra Silvertongue",
-  "NamePossessive": "Lyra Silvertongue's",
-  "Species": "Half-Elf",
-  "HomeLocation": "Silverport",
-  "CurrentLocation": "Silverport",
-  "Faction": "The Silent Coin",
-  "OwnedItems": {
-    "Lockpicks": 1,
-    "Merchant's Ledger": 1
-  },
-  "Role": "Merchant",
-  "Relations": [
-    {"Target": "The Traveler", "Favorability": -5},
-    {"Target": "The Silent Coin", "Favorability": 40},
-    {"Target": "The Iron Circle", "Favorability": 5},
-    {"Target": "Jasper Finn", "Favorability": 25},
-    {"Target": "Nyx", "Favorability": 20},
-    {"Target": "Silas Darkwater", "Favorability": 15},
-    {"Target": "Marcus Reed", "Favorability": -5},
-    {"Target": "Pippin Thistlefoot", "Favorability": 15}
-  ],
-  "NPCLog": []
-}
-Grimmok Bloodfist: {
-  "Name": "Grimmok Bloodfist",
-  "NamePossessive": "Grimmok Bloodfist's",
-  "Species": "Orc",
-  "HomeLocation": "Crimson Badlands",
-  "CurrentLocation": "Crimson Badlands",
-  "Faction": "Crimson Marauders",
-  "OwnedItems": {
-    "Steel Dagger": 1,
-    "Smoke Bomb": 2
-  },
-  "Role": "Mercenary",
-  "Relations": [
-    {"Target": "The Traveler", "Favorability": -15},
-    {"Target": "Crimson Marauders", "Favorability": 35},
-    {"Target": "Verdant Enclave", "Favorability": -50},
-    {"Target": "Chief Urgnak", "Favorability": 40},
-    {"Target": "Garrick", "Favorability": 25},
-    {"Target": "Mira", "Favorability": 20},
-    {"Target": "Elderon Greenscale", "Favorability": -40},
-    {"Target": "Kaelen Swiftarrow", "Favorability": -35},
-    {"Target": "Nyx", "Favorability": 5}
-  ],
-  "NPCLog": []
-}
-Pippin Thistlefoot: {
-  "Name": "Pippin Thistlefoot",
-  "NamePossessive": "Pippin Thistlefoot's",
-  "Species": "Halfling",
-  "HomeLocation": "Verdantia",
-  "CurrentLocation": "Verdantia",
-  "Faction": null,
-  "OwnedItems": {
-    "Cooking Spices": 2,
-    "Salted Meat": 5
-  },
-  "Role": "Innkeeper",
-  "Relations": [
-    {"Target": "The Traveler", "Favorability": 15},
-    {"Target": "The Iron Circle", "Favorability": 10},
-    {"Target": "Lyra Silvertongue", "Favorability": 15},
-    {"Target": "Barnaby Cole", "Favorability": 30},
-    {"Target": "Father Dominic", "Favorability": 20},
-    {"Target": "Flick", "Favorability": -5}
-  ],
-  "NPCLog": []
-}
-Seraphina Dawnseeker: {
-  "Name": "Seraphina Dawnseeker",
-  "NamePossessive": "Seraphina Dawnseeker's",
-  "Species": "Human",
-  "HomeLocation": "Verdantia",
-  "CurrentLocation": "Verdantia",
-  "Faction": null,
-  "OwnedItems": {
-    "Mage Robe": 1,
-    "Enchanted Amulet": 1
-  },
-  "Role": "Priest",
-  "Relations": [
-    {"Target": "The Traveler", "Favorability": 25},
-    {"Target": "Verdant Enclave", "Favorability": 20},
-    {"Target": "Father Dominic", "Favorability": 30},
-    {"Target": "Marcus Reed", "Favorability": 15},
-    {"Target": "Cyrus the Cursed", "Favorability": -10},
-    {"Target": "Madame Zephyra", "Favorability": -5}
-  ],
-  "NPCLog": []
-}
-Borin Ironfoot: {
-  "Name": "Borin Ironfoot",
-  "NamePossessive": "Borin Ironfoot's",
-  "Species": "Dwarf",
-  "HomeLocation": "Elderforge Mountain",
-  "CurrentLocation": "Elderforge Mountain",
-  "Faction": "The Keepers of the Forge",
-  "OwnedItems": {
-    "Iron Shield": 1,
-    "Chainmail Vest": 1
-  },
-  "Role": "GuardCaptain",
-  "Relations": [
-    {"Target": "The Traveler", "Favorability": 15},
-    {"Target": "The Keepers of the Forge", "Favorability": 45},
-    {"Target": "Durin Stonebrow", "Favorability": 30},
-    {"Target": "Thrain Coalbeard", "Favorability": 40},
-    {"Target": "Talia Ironvein", "Favorability": 35},
-    {"Target": "Grimmok Bloodfist", "Favorability": -15}
-  ],
-  "NPCLog": []
-}
-Sasha Voss: {
-  "Name": "Sasha Voss",
-  "NamePossessive": "Sasha Voss'",
-  "Species": "Human",
-  "HomeLocation": "Ironhold",
-  "CurrentLocation": "Ironhold",
-  "Faction": "The Iron Circle",
-  "OwnedItems": {
-    "Iron Longsword": 1,
-    "Traveling Cloak": 1
-  },
-  "Role": "Spy",
-  "Relations": [
-    {"Target": "The Traveler", "Favorability": 5},
-    {"Target": "The Iron Circle", "Favorability": 35},
-    {"Target": "The Silent Coin", "Favorability": -5},
-    {"Target": "Captain Valeria Holt", "Favorability": 30},
-    {"Target": "Marcus Reed", "Favorability": 20},
-    {"Target": "Nyx", "Favorability": -10},
-    {"Target": "Veronica Vane", "Favorability": -15}
-  ],
-  "NPCLog": []
-}
-Marcus Reed: {
-  "Name": "Marcus Reed",
-  "NamePossessive": "Marcus Reed's",
-  "Species": "Human",
-  "HomeLocation": "Ironhold",
-  "CurrentLocation": "Ironhold",
-  "Faction": "The Iron Circle",
-  "OwnedItems": {
-    "Iron Shield": 1,
-    "Salted Meat": 2
-  },
-  "Role": "GuardCaptain",
-  "Relations": [
-    {"Target": "The Traveler", "Favorability": 20},
-    {"Target": "The Iron Circle", "Favorability": 40},
-    {"Target": "Crimson Marauders", "Favorability": -25},
-    {"Target": "Captain Valeria Holt", "Favorability": 45},
-    {"Target": "Bram Heston", "Favorability": 20},
-    {"Target": "Roland the Stout", "Favorability": 25},
-    {"Target": "Garrick", "Favorability": -30}
-  ],
-  "NPCLog": []
-}
-Isolde: {
-  "Name": "Isolde",
-  "NamePossessive": "Isolde's",
-  "Species": "Human",
-  "HomeLocation": "Frostveil Tundra",
-  "CurrentLocation": "Frostveil Tundra",
-  "Faction": null,
-  "OwnedItems": {
-    "Health Potion": 3,
-    "Cooking Spices": 1
-  },
-  "Role": "Apothecary",
-  "Relations": [
-    {"Target": "The Traveler", "Favorability": 10},
-    {"Target": "Verdant Enclave", "Favorability": 15},
-    {"Target": "Elderon Greenscale", "Favorability": 20},
-    {"Target": "Vanya", "Favorability": 25},
-    {"Target": "Cyrus the Cursed", "Favorability": -20}
-  ],
-  "NPCLog": []
-}
-Thrain Coalbeard: {
-  "Name": "Thrain Coalbeard",
-  "NamePossessive": "Thrain Coalbeard's",
-  "Species": "Dwarf",
-  "HomeLocation": "Elderforge Mountain",
-  "CurrentLocation": "Elderforge Mountain",
-  "Faction": "The Keepers of the Forge",
-  "OwnedItems": {
-    "Obsidian Shard": 10,
-    "Dwarven Ale": 2
-  },
-  "Role": "Merchant",
-  "Relations": [
-    {"Target": "The Traveler", "Favorability": 10},
-    {"Target": "The Keepers of the Forge", "Favorability": 35},
-    {"Target": "The Silent Coin", "Favorability": 20},
-    {"Target": "Durin Stonebrow", "Favorability": 35},
-    {"Target": "Lyra Silvertongue", "Favorability": 15},
-    {"Target": "Grizzle Geargrinder", "Favorability": 30}
-  ],
-  "NPCLog": []
-}
-Elara Moonshadow: {
-  "Name": "Elara Moonshadow",
-  "NamePossessive": "Elara Moonshadow's",
-  "Species": "Elf",
-  "HomeLocation": "Whispering Woods",
-  "CurrentLocation": "Whispering Woods",
-  "Faction": "Verdant Enclave",
-  "OwnedItems": {
-    "Mana Vial": 2,
-    "Glowdust": 5
-  },
-  "Role": "Wizard",
-  "Relations": [
-    {"Target": "The Traveler", "Favorability": 30},
-    {"Target": "Verdant Enclave", "Favorability": 40},
-    {"Target": "Elderon Greenscale", "Favorability": 35},
-    {"Target": "Kaelen Swiftarrow", "Favorability": 40},
-    {"Target": "Whispering Willow", "Favorability": 25},
-    {"Target": "Madame Zephyra", "Favorability": 15}
-  ],
-  "NPCLog": []
-}
-Roric: {
-  "Name": "Roric",
-  "NamePossessive": "Roric's",
-  "Species": "Human",
-  "HomeLocation": "Sunstone Oasis",
-  "CurrentLocation": "Sunstone Oasis",
-  "Faction": null,
-  "OwnedItems": {
-    "Fresh Water": 3,
-    "Salted Meat": 2
-  },
-  "Role": "Hunter",
-  "Relations": [
-    {"Target": "The Traveler", "Favorability": 0},
-    {"Target": "Crimson Marauders", "Favorability": -15},
-    {"Target": "Garrick", "Favorability": -20},
-    {"Target": "Anya", "Favorability": 15}
-  ],
-  "NPCLog": []
-}
-Gretta: {
-  "Name": "Gretta",
-  "NamePossessive": "Gretta's",
-  "Species": "Human",
-  "HomeLocation": "Ironhold",
-  "CurrentLocation": "Ironhold",
-  "Faction": null,
-  "OwnedItems": {
-    "Copper Coin": 25,
-    "Elven Bread": 2
-  },
-  "Role": "Farmer",
-  "Relations": [
-    {"Target": "The Traveler", "Favorability": 5},
-    {"Target": "The Iron Circle", "Favorability": 15},
-    {"Target": "Bram Heston", "Favorability": 20},
-    {"Target": "Barnaby Cole", "Favorability": 10}
-  ],
-  "NPCLog": []
-}
-Jasper Finn: {
-  "Name": "Jasper Finn",
-  "NamePossessive": "Jasper Finn's",
-  "Species": "Halfling",
-  "HomeLocation": "Silverport",
-  "CurrentLocation": "Silverport",
-  "Faction": "The Silent Coin",
-  "OwnedItems": {
-    "Lockpicks": 1,
-    "Silver Mark": 10
-  },
-  "Role": "Thief",
-  "Relations": [
-    {"Target": "The Traveler", "Favorability": 0},
-    {"Target": "The Silent Coin", "Favorability": 30},
-    {"Target": "Lyra Silvertongue", "Favorability": 25},
-    {"Target": "Nyx", "Favorability": 20},
-    {"Target": "Flick", "Favorability": 15},
-    {"Target": "Marcus Reed", "Favorability": -10}
-  ],
-  "NPCLog": []
-}
-Nyx: {
-  "Name": "Nyx",
-  "NamePossessive": "Nyx's",
-  "Species": "Goblin",
-  "HomeLocation": "Shadowfen Swamp",
-  "CurrentLocation": "Silverport",
-  "Faction": "The Silent Coin",
-  "OwnedItems": {
-    "Smoke Bomb": 3,
-    "Steel Dagger": 1
-  },
-  "Role": "Spy",
-  "Relations": [
-    {"Target": "The Traveler", "Favorability": -10},
-    {"Target": "The Silent Coin", "Favorability": 35},
-    {"Target": "Crimson Marauders", "Favorability": 10},
-    {"Target": "Lyra Silvertongue", "Favorability": 20},
-    {"Target": "Silas Darkwater", "Favorability": 25},
-    {"Target": "Sasha Voss", "Favorability": -10}
-  ],
-  "NPCLog": []
-}
-Captain Valeria Holt: {
-  "Name": "Captain Valeria Holt",
-  "NamePossessive": "Captain Valeria Holt's",
-  "Species": "Human",
-  "HomeLocation": "Ironhold",
-  "CurrentLocation": "Ironhold",
-  "Faction": "The Iron Circle",
-  "OwnedItems": {
-    "Iron Longsword": 1,
-    "Iron Shield": 1
-  },
-  "Role": "GuardCaptain",
-  "Relations": [
-    {"Target": "The Traveler", "Favorability": 25},
-    {"Target": "The Iron Circle", "Favorability": 50},
-    {"Target": "Crimson Marauders", "Favorability": -40},
-    {"Target": "Marcus Reed", "Favorability": 45},
-    {"Target": "Sasha Voss", "Favorability": 30},
-    {"Target": "Bram Heston", "Favorability": 20},
-    {"Target": "Chief Urgnak", "Favorability": -45}
-  ],
-  "NPCLog": []
-}
-Barnaby Cole: {
-  "Name": "Barnaby Cole",
-  "NamePossessive": "Barnaby Cole's",
-  "Species": "Human",
-  "HomeLocation": "Verdantia",
-  "CurrentLocation": "Verdantia",
-  "Faction": null,
-  "OwnedItems": {
-    "Cooking Spices": 3,
-    "Dwarven Ale": 5
-  },
-  "Role": "Bard",
-  "Relations": [
-    {"Target": "The Traveler", "Favorability": 20},
-    {"Target": "The Silent Coin", "Favorability": 5},
-    {"Target": "Pippin Thistlefoot", "Favorability": 30},
-    {"Target": "Zargoth the Melodious", "Favorability": 25},
-    {"Target": "Flick", "Favorability": 0}
-  ],
-  "NPCLog": []
-}
-Whispering Willow: {
-  "Name": "Whispering Willow",
-  "NamePossessive": "Whispering Willow's",
-  "Species": "Elf",
-  "HomeLocation": "Whispering Woods",
-  "CurrentLocation": "Whispering Woods",
-  "Faction": "Verdant Enclave",
-  "OwnedItems": {
-    "Elven Bread": 5,
-    "Health Potion": 2
-  },
-  "Role": "Ranger",
-  "Relations": [
-    {"Target": "The Traveler", "Favorability": 25},
-    {"Target": "Verdant Enclave", "Favorability": 35},
-    {"Target": "Kaelen Swiftarrow", "Favorability": 30},
-    {"Target": "Elderon Greenscale", "Favorability": 20},
-    {"Target": "Lysander", "Favorability": 35},
-    {"Target": "Grimmok Bloodfist", "Favorability": -35}
-  ],
-  "NPCLog": []
-}
-Zargoth the Melodious: {
-  "Name": "Zargoth the Melodious",
-  "NamePossessive": "Zargoth the Melodious'",
-  "Species": "Orc",
-  "HomeLocation": "Crimson Badlands",
-  "CurrentLocation": "Verdantia",
-  "Faction": null,
-  "OwnedItems": {
-    "Traveling Cloak": 1,
-    "Gold Crown": 5
-  },
-  "Role": "Bard",
-  "Relations": [
-    {"Target": "The Traveler", "Favorability": 15},
-    {"Target": "Crimson Marauders", "Favorability": 10},
-    {"Target": "Barnaby Cole", "Favorability": 25},
-    {"Target": "Pippin Thistlefoot", "Favorability": 20},
-    {"Target": "Grimmok Bloodfist", "Favorability": 15}
-  ],
-  "NPCLog": []
-}
-Father Dominic: {
-  "Name": "Father Dominic",
-  "NamePossessive": "Father Dominic's",
-  "Species": "Human",
-  "HomeLocation": "Verdantia",
-  "CurrentLocation": "Verdantia",
-  "Faction": null,
-  "OwnedItems": {
-    "Enchanted Amulet": 1,
-    "Ancient Grimoire": 1
-  },
-  "Role": "Priest",
-  "Relations": [
-    {"Target": "The Traveler", "Favorability": 20},
-    {"Target": "Verdant Enclave", "Favorability": 20},
-    {"Target": "Seraphina Dawnseeker", "Favorability": 30},
-    {"Target": "Cyrus the Cursed", "Favorability": -25}
-  ],
-  "NPCLog": []
-}
-Helga Giantbone: {
-  "Name": "Helga Giantbone",
-  "NamePossessive": "Helga Giantbone's",
-  "Species": "Half-Elf",
-  "HomeLocation": "Frostveil Tundra",
-  "CurrentLocation": "Frostveil Tundra",
-  "Faction": null,
-  "OwnedItems": {
-    "Bear Trap": 2,
-    "Salted Meat": 10
-  },
-  "Role": "Hunter",
-  "Relations": [
-    {"Target": "The Traveler", "Favorability": 5},
-    {"Target": "The Iron Circle", "Favorability": 10},
-    {"Target": "Isolde", "Favorability": 20},
-    {"Target": "Vanya", "Favorability": 15},
-    {"Target": "Mira", "Favorability": -15}
-  ],
-  "NPCLog": []
-}
-Finnian: {
-  "Name": "Finnian",
-  "NamePossessive": "Finnian's",
-  "Species": "Halfling",
-  "HomeLocation": "Silverport",
-  "CurrentLocation": "Silverport",
-  "Faction": null,
-  "OwnedItems": {
-    "Silver Mark": 5,
-    "Copper Coin": 50
-  },
-  "Role": "Fisherman",
-  "Relations": [
-    {"Target": "The Traveler", "Favorability": 10},
-    {"Target": "The Silent Coin", "Favorability": 0},
-    {"Target": "Pearl", "Favorability": 25},
-    {"Target": "Silas Darkwater", "Favorability": -5}
-  ],
-  "NPCLog": []
-}
-Click-Clack: {
-  "Name": "Click-Clack",
-  "NamePossessive": "Click-Clack's",
-  "Species": "Goblin",
-  "HomeLocation": "The Sinking Marshes",
-  "CurrentLocation": "The Sinking Marshes",
-  "Faction": null,
-  "OwnedItems": {
-    "Lockpicks": 1,
-    "Glowdust": 10
-  },
-  "Role": "Alchemist",
-  "Relations": [
-    {"Target": "The Traveler", "Favorability": -15},
-    {"Target": "Crimson Marauders", "Favorability": 5},
-    {"Target": "Nyx", "Favorability": 15},
-    {"Target": "Squeak", "Favorability": 20},
-    {"Target": "Elderon Greenscale", "Favorability": -20}
-  ],
-  "NPCLog": []
-}
-Boulder: {
-  "Name": "Boulder",
-  "NamePossessive": "Boulder's",
-  "Species": "Troll",
-  "HomeLocation": "Elderforge Mount</t>
-  </si>
-  <si>
     <t xml:space="preserve">## ENUM DATA
 {
   "Types": {
@@ -18290,6 +17282,3066 @@
     {"Target": "Fiora", "Favorability": 30},
     {"Target": "Wren", "Favorability": 25},
     {"Target": "Vex", "Favorability": </t>
+  </si>
+  <si>
+    <t>## ENUM DATA
+{
+  "Types": {
+    "ItemTypes": ["Weapon", "Armor", "Potion", "Ingredient", "Key", "Artifact", "Currency", "Scroll", "Tool", "Food"],
+    "QuestTypes": ["AttackThreateningEntities", "RecoverStolenItem", "GuardEntity", "AttackEnemy", "StealStuff", "KillEnemies"],
+    "EventTypes": ["Ambush", "Discovery", "Betrayal", "Alliance", "TradeRouteOpened", "ResourceDepleted", "Theft", "Rescue", "CraftingBreakthrough", "Eclipse"],
+    "RelationshipLevels": {"Sworn Enemy" : -50, "Enemy" : -30, "Hated" : -15, "Disliked" : -5, "Neutral" : 0, "Friendly" : 5, "Friend" : 15, "Ally" : 30, "Sworn Ally" : 50}
+  },
+  "Lists": {
+    "Species": ["Human", "Elf", "Dwarf", "Orc", "Halfling", "Lizardfolk", "Goblin", "Troll", "Gnome", "Fae"],
+    "Roles": ["Innkeeper", "Blacksmith", "Merchant", "GuardCaptain", "Apothecary", "Thief", "Wizard", "Ranger", "Bard", "Priest", "Alchemist", "Farmer", "Mercenary", "Noble", "Beggar", "Spy", "ShipCaptain", "Librarian", "Hunter", "Miner"],
+    "Locations": ["Silverwood", "Ironhold", "Ravenport", "SunkenRuins", "Embermaw", "VerdantGlade", "TheSpire", "Dreadmarsh", "AzureCoast", "FrostfangPeak"],
+    "Factions": ["SilverwoodCouncil", "IronholdConglomerate", "RavenportSyndicate", "EmbermawClan", "OrderOfTheSpire"],
+    "Enemies": ["ShadowStalker", "RazorbackBoar", "VenomousSkitterer", "FrostWraith", "EmberElemental", "DrownedSailor", "CaveTroll", "GoblinScavenger", "DireWolf", "GiantSpider", "SkeletalWarrior", "HarpyScreecher", "Mudcrab", "BanditMarauder", "CorruptedDryad", "LavaSnail", "StormHawk", "PlagueRat", "StoneGolem", "DeepOneHybrid"],
+    "Items": ["IronSword", "SteelDagger", "LeatherArmor", "HealthPotion", "ManaElixir", "LockpickSet", "SilverRing", "AncientCoin", "DragonScale", "GhostOrchid", "IronOre", "SturdyShield", "EnchantedStaff", "ThievesGuildCharm", "ShipManifest", "NobleSignet", "ObsidianArrow", "Rations", "Waterskin", "BlackPearl", "GoblinEar", "TrollFat", "FireSalt", "FrostMirror", "CrystalShard", "SpellScrollLight", "GrapplingHook", "MiningPick", "FishingRod", "Emberbloom"],
+    "NPCs": ["KaelenSilverwood", "ThaliaIronfoot", "BorinCoppervein", "CaptainRook", "ElaraMoonshadow", "GrizzleGearspark", "SeraphinaVex", "UrgathBonebreaker", "MiloProudfoot", "SszikVess", "BrotherAlaric", "MadamVivienne", "OrinSteelhand", "LilyRosewater", "DariusBlack", "YgritteFrostbane", "PercivalRustbucket", "NyxShadowmere", "GornHammerfall", "FizzwickTinkertop", "SeleneStarweaver", "BartholomewReed", "RaskulGnarltooth", "MorganaDreadveil", "FinnianSwift", "GretaStonebrew", "ValeriusCorvus", "EldrinOakenshield", "QuinnSilverton", "ZaraNightshade", "TiberiusGrimm", "IsoldeMistwalker", "GrummokSkullcrusher", "PennyHoneytongue", "CassianVale", "VanyaStormrider", "DurinIronmantle", "LyraQuickstep", "MalachaiGraves", "OpalStardust", "RoricBoulderback", "JasperWindleaf", "SableFell", "HildaBarleybrew", "CyrusVance", "ElysiaDawnseeker", "GrobnikSneakwhistle", "MiraFireheart", "AldricTrueblade", "BelladonnaShade", "WrenFeatherdown", "ViktorDragomir", "NalaSandskimmer", "FergusMcBrick"],
+    "Player": ["Vesper"]
+  }
+}
+;
+### ITEM DATA
+IronSword: { 
+  "Type": "Weapon", 
+  "Name": "IronSword", 
+  "NameSingular": "iron sword", 
+  "NamePlural": "iron swords",
+  "NamePossessiveSingular": "iron sword's",
+  "NamePossessivePlural": "iron swords'",
+  "IndefiniteArticle": "an",
+  "IndefiniteArticleCaps": "An"
+}
+SteelDagger: { 
+  "Type": "Weapon", 
+  "Name": "SteelDagger", 
+  "NameSingular": "steel dagger", 
+  "NamePlural": "steel daggers",
+  "NamePossessiveSingular": "steel dagger's",
+  "NamePossessivePlural": "steel daggers'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+LeatherArmor: { 
+  "Type": "Armor", 
+  "Name": "LeatherArmor", 
+  "NameSingular": "leather tunic", 
+  "NamePlural": "leather tunics",
+  "NamePossessiveSingular": "leather tunic's",
+  "NamePossessivePlural": "leather tunics'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+HealthPotion: { 
+  "Type": "Potion", 
+  "Name": "HealthPotion", 
+  "NameSingular": "health potion", 
+  "NamePlural": "health potions",
+  "NamePossessiveSingular": "health potion's",
+  "NamePossessivePlural": "health potions'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+ManaElixir: { 
+  "Type": "Potion", 
+  "Name": "ManaElixir", 
+  "NameSingular": "mana elixir", 
+  "NamePlural": "mana elixirs",
+  "NamePossessiveSingular": "mana elixir's",
+  "NamePossessivePlural": "mana elixirs'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+LockpickSet: { 
+  "Type": "Tool", 
+  "Name": "LockpickSet", 
+  "NameSingular": "lockpick set", 
+  "NamePlural": "lockpick sets",
+  "NamePossessiveSingular": "lockpick set's",
+  "NamePossessivePlural": "lockpick sets'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+SilverRing: { 
+  "Type": "Artifact", 
+  "Name": "SilverRing", 
+  "NameSingular": "silver ring", 
+  "NamePlural": "silver rings",
+  "NamePossessiveSingular": "silver ring's",
+  "NamePossessivePlural": "silver rings'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+AncientCoin: { 
+  "Type": "Currency", 
+  "Name": "AncientCoin", 
+  "NameSingular": "ancient coin", 
+  "NamePlural": "ancient coins",
+  "NamePossessiveSingular": "ancient coin's",
+  "NamePossessivePlural": "ancient coins'",
+  "IndefiniteArticle": "an",
+  "IndefiniteArticleCaps": "An"
+}
+DragonScale: { 
+  "Type": "Ingredient", 
+  "Name": "DragonScale", 
+  "NameSingular": "dragon scale", 
+  "NamePlural": "dragon scales",
+  "NamePossessiveSingular": "dragon scale's",
+  "NamePossessivePlural": "dragon scales'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+GhostOrchid: { 
+  "Type": "Ingredient", 
+  "Name": "GhostOrchid", 
+  "NameSingular": "ghost orchid", 
+  "NamePlural": "ghost orchids",
+  "NamePossessiveSingular": "ghost orchid's",
+  "NamePossessivePlural": "ghost orchids'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+IronOre: { 
+  "Type": "Ingredient", 
+  "Name": "IronOre", 
+  "NameSingular": "iron ore", 
+  "NamePlural": "iron ores",
+  "NamePossessiveSingular": "iron ore's",
+  "NamePossessivePlural": "iron ores'",
+  "IndefiniteArticle": "an",
+  "IndefiniteArticleCaps": "An"
+}
+SturdyShield: { 
+  "Type": "Armor", 
+  "Name": "SturdyShield", 
+  "NameSingular": "sturdy shield", 
+  "NamePlural": "sturdy shields",
+  "NamePossessiveSingular": "sturdy shield's",
+  "NamePossessivePlural": "sturdy shields'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+EnchantedStaff: { 
+  "Type": "Weapon", 
+  "Name": "EnchantedStaff", 
+  "NameSingular": "enchanted staff", 
+  "NamePlural": "enchanted staves",
+  "NamePossessiveSingular": "enchanted staff's",
+  "NamePossessivePlural": "enchanted staves'",
+  "IndefiniteArticle": "an",
+  "IndefiniteArticleCaps": "An"
+}
+ThievesGuildCharm: { 
+  "Type": "Artifact", 
+  "Name": "ThievesGuildCharm", 
+  "NameSingular": "thieves' guild charm", 
+  "NamePlural": "thieves' guild charms",
+  "NamePossessiveSingular": "thieves' guild charm's",
+  "NamePossessivePlural": "thieves' guild charms'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+ShipManifest: { 
+  "Type": "Key", 
+  "Name": "ShipManifest", 
+  "NameSingular": "ship manifest", 
+  "NamePlural": "ship manifests",
+  "NamePossessiveSingular": "ship manifest's",
+  "NamePossessivePlural": "ship manifests'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+NobleSignet: { 
+  "Type": "Key", 
+  "Name": "NobleSignet", 
+  "NameSingular": "noble's signet ring", 
+  "NamePlural": "nobles' signet rings",
+  "NamePossessiveSingular": "noble's signet ring's",
+  "NamePossessivePlural": "nobles' signet rings'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+ObsidianArrow: { 
+  "Type": "Weapon", 
+  "Name": "ObsidianArrow", 
+  "NameSingular": "obsidian arrow", 
+  "NamePlural": "obsidian arrows",
+  "NamePossessiveSingular": "obsidian arrow's",
+  "NamePossessivePlural": "obsidian arrows'",
+  "IndefiniteArticle": "an",
+  "IndefiniteArticleCaps": "An"
+}
+Rations: { 
+  "Type": "Food", 
+  "Name": "Rations", 
+  "NameSingular": "ration pack", 
+  "NamePlural": "ration packs",
+  "NamePossessiveSingular": "ration pack's",
+  "NamePossessivePlural": "ration packs'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+Waterskin: { 
+  "Type": "Tool", 
+  "Name": "Waterskin", 
+  "NameSingular": "waterskin", 
+  "NamePlural": "waterskins",
+  "NamePossessiveSingular": "waterskin's",
+  "NamePossessivePlural": "waterskins'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+BlackPearl: { 
+  "Type": "Artifact", 
+  "Name": "BlackPearl", 
+  "NameSingular": "black pearl", 
+  "NamePlural": "black pearls",
+  "NamePossessiveSingular": "black pearl's",
+  "NamePossessivePlural": "black pearls'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+GoblinEar: { 
+  "Type": "Ingredient", 
+  "Name": "GoblinEar", 
+  "NameSingular": "goblin ear", 
+  "NamePlural": "goblin ears",
+  "NamePossessiveSingular": "goblin ear's",
+  "NamePossessivePlural": "goblin ears'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+TrollFat: { 
+  "Type": "Ingredient", 
+  "Name": "TrollFat", 
+  "NameSingular": "troll fat", 
+  "NamePlural": "troll fats",
+  "NamePossessiveSingular": "troll fat's",
+  "NamePossessivePlural": "troll fats'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+FireSalt: { 
+  "Type": "Ingredient", 
+  "Name": "FireSalt", 
+  "NameSingular": "fire salt", 
+  "NamePlural": "fire salts",
+  "NamePossessiveSingular": "fire salt's",
+  "NamePossessivePlural": "fire salts'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+FrostMirror: { 
+  "Type": "Artifact", 
+  "Name": "FrostMirror", 
+  "NameSingular": "frost mirror", 
+  "NamePlural": "frost mirrors",
+  "NamePossessiveSingular": "frost mirror's",
+  "NamePossessivePlural": "frost mirrors'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+CrystalShard: { 
+  "Type": "Ingredient", 
+  "Name": "CrystalShard", 
+  "NameSingular": "crystal shard", 
+  "NamePlural": "crystal shards",
+  "NamePossessiveSingular": "crystal shard's",
+  "NamePossessivePlural": "crystal shards'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+SpellScrollLight: { 
+  "Type": "Scroll", 
+  "Name": "SpellScrollLight", 
+  "NameSingular": "scroll of light", 
+  "NamePlural": "scrolls of light",
+  "NamePossessiveSingular": "scroll of light's",
+  "NamePossessivePlural": "scrolls of light's",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+GrapplingHook: { 
+  "Type": "Tool", 
+  "Name": "GrapplingHook", 
+  "NameSingular": "grappling hook", 
+  "NamePlural": "grappling hooks",
+  "NamePossessiveSingular": "grappling hook's",
+  "NamePossessivePlural": "grappling hooks'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+MiningPick: { 
+  "Type": "Tool", 
+  "Name": "MiningPick", 
+  "NameSingular": "mining pick", 
+  "NamePlural": "mining picks",
+  "NamePossessiveSingular": "mining pick's",
+  "NamePossessivePlural": "mining picks'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+FishingRod: { 
+  "Type": "Tool", 
+  "Name": "FishingRod", 
+  "NameSingular": "fishing rod", 
+  "NamePlural": "fishing rods",
+  "NamePossessiveSingular": "fishing rod's",
+  "NamePossessivePlural": "fishing rods'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+Emberbloom: { 
+  "Type": "Ingredient", 
+  "Name": "Emberbloom", 
+  "NameSingular": "emberbloom flower", 
+  "NamePlural": "emberbloom flowers",
+  "NamePossessiveSingular": "emberbloom flower's",
+  "NamePossessivePlural": "emberbloom flowers'",
+  "IndefiniteArticle": "an",
+  "IndefiniteArticleCaps": "An"
+}
+;
+## GAME STATE DATA
+### FACTION DATA
+SilverwoodCouncil: {
+  "Name": "SilverwoodCouncil", 
+  "NameDefinitive": "the Silverwood Council",
+  "NameDefinitiveCaps": "The Silverwood Council",
+  "NamePossessive": "Silverwood Council's",
+  "NameDefinitivePossessive": "the Silverwood Council's",
+  "NameDefinitivePossessiveCaps": "The Silverwood Council's",
+  "DefaultLocation": "Silverwood",
+  "Relations": [
+    {"Target": "Vesper", "Favorability": 15},
+    {"Target": "IronholdConglomerate", "Favorability": -5},
+    {"Target": "RavenportSyndicate", "Favorability": -30},
+    {"Target": "EmbermawClan", "Favorability": -15},
+    {"Target": "OrderOfTheSpire", "Favorability": 5}
+  ],
+  "Members": ["KaelenSilverwood", "ElaraMoonshadow", "BrotherAlaric", "SeleneStarweaver", "AldricTrueblade", "ElysiaDawnseeker", "FinnianSwift", "IsoldeMistwalker", "JasperWindleaf", "WrenFeatherdown"],
+  "Treasury": {
+    "IronSword": 5, "LeatherArmor": 3, "HealthPotion": 10, "Rations": 20, "SpellScrollLight": 2, "AncientCoin": 150
+  },
+  "FactionLog": []
+}
+IronholdConglomerate: {
+  "Name": "IronholdConglomerate", 
+  "NameDefinitive": "the Ironhold Conglomerate",
+  "NameDefinitiveCaps": "The Ironhold Conglomerate",
+  "NamePossessive": "Ironhold Conglomerate's",
+  "NameDefinitivePossessive": "the Ironhold Conglomerate's",
+  "NameDefinitivePossessiveCaps": "The Ironhold Conglomerate's",
+  "DefaultLocation": "Ironhold",
+  "Relations": [
+    {"Target": "Vesper", "Favorability": -5},
+    {"Target": "SilverwoodCouncil", "Favorability": -5},
+    {"Target": "RavenportSyndicate", "Favorability": -15},
+    {"Target": "EmbermawClan", "Favorability": 30},
+    {"Target": "OrderOfTheSpire", "Favorability": 0}
+  ],
+  "Members": ["ThaliaIronfoot", "BorinCoppervein", "GornHammerfall", "DurinIronmantle", "RoricBoulderback", "HildaBarleybrew", "FergusMcBrick", "GretaStonebrew", "OrinSteelhand", "MiraFireheart"],
+  "Treasury": {
+    "IronOre": 50, "MiningPick": 5, "SturdyShield": 3, "IronSword": 2, "HealthPotion": 5, "AncientCoin": 500
+  },
+  "FactionLog": []
+}
+RavenportSyndicate: {
+  "Name": "RavenportSyndicate", 
+  "NameDefinitive": "the Ravenport Syndicate",
+  "NameDefinitiveCaps": "The Ravenport Syndicate",
+  "NamePossessive": "Ravenport Syndicate's",
+  "NameDefinitivePossessive": "the Ravenport Syndicate's",
+  "NameDefinitivePossessiveCaps": "The Ravenport Syndicate's",
+  "DefaultLocation": "Ravenport",
+  "Relations": [
+    {"Target": "Vesper", "Favorability": 30},
+    {"Target": "SilverwoodCouncil", "Favorability": -30},
+    {"Target": "IronholdConglomerate", "Favorability": -15},
+    {"Target": "EmbermawClan", "Favorability": -50},
+    {"Target": "OrderOfTheSpire", "Favorability": -15}
+  ],
+  "Members": ["CaptainRook", "SeraphinaVex", "DariusBlack", "NyxShadowmere", "MorganaDreadveil", "QuinnSilverton", "ZaraNightshade", "MalachaiGraves", "SableFell", "BelladonnaShade", "GrobnikSneakwhistle"],
+  "Treasury": {
+    "LockpickSet": 10, "SteelDagger": 8, "ThievesGuildCharm": 4, "BlackPearl": 7, "HealthPotion": 3, "AncientCoin": 750
+  },
+  "FactionLog": []
+}
+EmbermawClan: {
+  "Name": "EmbermawClan", 
+  "NameDefinitive": "the Embermaw Clan",
+  "NameDefinitiveCaps": "The Embermaw Clan",
+  "NamePossessive": "Embermaw Clan's",
+  "NameDefinitivePossessive": "the Embermaw Clan's",
+  "NameDefinitivePossessiveCaps": "The Embermaw Clan's",
+  "DefaultLocation": "Embermaw",
+  "Relations": [
+    {"Target": "Vesper", "Favorability": -15},
+    {"Target": "SilverwoodCouncil", "Favorability": -15},
+    {"Target": "IronholdConglomerate", "Favorability": 30},
+    {"Target": "RavenportSyndicate", "Favorability": -50},
+    {"Target": "OrderOfTheSpire", "Favorability": -30}
+  ],
+  "Members": ["UrgathBonebreaker", "RaskulGnarltooth", "GrummokSkullcrusher", "ViktorDragomir", "YgritteFrostbane", "SszikVess"],
+  "Treasury": {
+    "FireSalt": 20, "ObsidianArrow": 30, "Emberbloom": 15, "TrollFat": 5, "Rations": 10, "AncientCoin": 200
+  },
+  "FactionLog": []
+}
+OrderOfTheSpire: {
+  "Name": "OrderOfTheSpire", 
+  "NameDefinitive": "the Order of the Spire",
+  "NameDefinitiveCaps": "The Order of the Spire",
+  "NamePossessive": "Order of the Spire's",
+  "NameDefinitivePossessive": "the Order of the Spire's",
+  "NameDefinitivePossessiveCaps": "The Order of the Spire's",
+  "DefaultLocation": "TheSpire",
+  "Relations": [
+    {"Target": "Vesper", "Favorability": 5},
+    {"Target": "SilverwoodCouncil", "Favorability": 5},
+    {"Target": "IronholdConglomerate", "Favorability": 0},
+    {"Target": "RavenportSyndicate", "Favorability": -15},
+    {"Target": "EmbermawClan", "Favorability": -30}
+  ],
+  "Members": ["MadamVivienne", "ValeriusCorvus", "TiberiusGrimm", "VanyaStormrider", "OpalStardust", "EldrinOakenshield", "CyrusVance", "NalaSandskimmer", "PercivalRustbucket"],
+  "Treasury": {
+    "ManaElixir": 10, "EnchantedStaff": 2, "CrystalShard": 8, "SpellScrollLight": 5, "FrostMirror": 1, "AncientCoin": 300
+  },
+  "FactionLog": []
+}
+;
+### NPC DATA
+KaelenSilverwood: {
+  "Name": "KaelenSilverwood",
+  "NamePossessive": "Kaelen Silverwood's",
+  "Species": "Elf",
+  "HomeLocation": "Silverwood",
+  "CurrentLocation": "Silverwood",
+  "Faction": "SilverwoodCouncil",
+  "OwnedItems": {
+    "IronSword": 1, "LeatherArmor": 1, "AncientCoin": 25
+  },
+  "Role": "Ranger",
+  "Relations": [
+    {"Target": "Vesper", "Favorability": 25},
+    {"Target": "SilverwoodCouncil", "Favorability": 40},
+    {"Target": "IronholdConglomerate", "Favorability": -10},
+    {"Target": "ElaraMoonshadow", "Favorability": 35},
+    {"Target": "ThaliaIronfoot", "Favorability": -15},
+    {"Target": "BrotherAlaric", "Favorability": 20},
+    {"Target": "CaptainRook", "Favorability": -40}
+  ],
+  "NPCLog": []
+}
+ThaliaIronfoot: {
+  "Name": "ThaliaIronfoot",
+  "NamePossessive": "Thalia Ironfoot's",
+  "Species": "Dwarf",
+  "HomeLocation": "Ironhold",
+  "CurrentLocation": "Ironhold",
+  "Faction": "IronholdConglomerate",
+  "OwnedItems": {
+    "MiningPick": 1, "IronOre": 15, "SturdyShield": 1
+  },
+  "Role": "Miner",
+  "Relations": [
+    {"Target": "Vesper", "Favorability": -10},
+    {"Target": "IronholdConglomerate", "Favorability": 45},
+    {"Target": "SilverwoodCouncil", "Favorability": -5},
+    {"Target": "BorinCoppervein", "Favorability": 30},
+    {"Target": "KaelenSilverwood", "Favorability": -15},
+    {"Target": "UrgathBonebreaker", "Favorability": 25}
+  ],
+  "NPCLog": []
+}
+BorinCoppervein: {
+  "Name": "BorinCoppervein",
+  "NamePossessive": "Borin Coppervein's",
+  "Species": "Dwarf",
+  "HomeLocation": "Ironhold",
+  "CurrentLocation": "Ironhold",
+  "Faction": "IronholdConglomerate",
+  "OwnedItems": {
+    "IronSword": 1, "HealthPotion": 2, "AncientCoin": 50
+  },
+  "Role": "Blacksmith",
+  "Relations": [
+    {"Target": "Vesper", "Favorability": 10},
+    {"Target": "IronholdConglomerate", "Favorability": 35},
+    {"Target": "EmbermawClan", "Favorability": 15},
+    {"Target": "ThaliaIronfoot", "Favorability": 30},
+    {"Target": "GornHammerfall", "Favorability": 40},
+    {"Target": "GrizzleGearspark", "Favorability": -20}
+  ],
+  "NPCLog": []
+}
+CaptainRook: {
+  "Name": "CaptainRook",
+  "NamePossessive": "Captain Rook's",
+  "Species": "Human",
+  "HomeLocation": "Ravenport",
+  "CurrentLocation": "AzureCoast",
+  "Faction": "RavenportSyndicate",
+  "OwnedItems": {
+    "SteelDagger": 1, "ShipManifest": 1, "BlackPearl": 2
+  },
+  "Role": "ShipCaptain",
+  "Relations": [
+    {"Target": "Vesper", "Favorability": 35},
+    {"Target": "RavenportSyndicate", "Favorability": 50},
+    {"Target": "SilverwoodCouncil", "Favorability": -35},
+    {"Target": "SeraphinaVex", "Favorability": 40},
+    {"Target": "DariusBlack", "Favorability": 25},
+    {"Target": "KaelenSilverwood", "Favorability": -40},
+    {"Target": "MadamVivienne", "Favorability": -25}
+  ],
+  "NPCLog": []
+}
+ElaraMoonshadow: {
+  "Name": "ElaraMoonshadow",
+  "NamePossessive": "Elara Moonshadow's",
+  "Species": "Elf",
+  "HomeLocation": "Silverwood",
+  "CurrentLocation": "Silverwood",
+  "Faction": "SilverwoodCouncil",
+  "OwnedItems": {
+    "EnchantedStaff": 1, "ManaElixir": 3, "CrystalShard": 2
+  },
+  "Role": "Wizard",
+  "Relations": [
+    {"Target": "Vesper", "Favorability": 15},
+    {"Target": "SilverwoodCouncil", "Favorability": 45},
+    {"Target": "OrderOfTheSpire", "Favorability": 10},
+    {"Target": "KaelenSilverwood", "Favorability": 35},
+    {"Target": "SeleneStarweaver", "Favorability": 30},
+    {"Target": "MadamVivienne", "Favorability": -5}
+  ],
+  "NPCLog": []
+}
+GrizzleGearspark: {
+  "Name": "GrizzleGearspark",
+  "NamePossessive": "Grizzle Gearspark's",
+  "Species": "Gnome",
+  "HomeLocation": "Ironhold",
+  "CurrentLocation": "Ironhold",
+  "Faction": "IronholdConglomerate",
+  "OwnedItems": {
+    "LockpickSet": 1, "GrapplingHook": 1, "FireSalt": 5
+  },
+  "Role": "Merchant",
+  "Relations": [
+    {"Target": "Vesper", "Favorability": 5},
+    {"Target": "IronholdConglomerate", "Favorability": 20},
+    {"Target": "RavenportSyndicate", "Favorability": -5},
+    {"Target": "BorinCoppervein", "Favorability": -20},
+    {"Target": "FizzwickTinkertop", "Favorability": 25},
+    {"Target": "PennyHoneytongue", "Favorability": 15}
+  ],
+  "NPCLog": []
+}
+SeraphinaVex: {
+  "Name": "SeraphinaVex",
+  "NamePossessive": "Seraphina Vex's",
+  "Species": "Human",
+  "HomeLocation": "Ravenport",
+  "CurrentLocation": "Ravenport",
+  "Faction": "RavenportSyndicate",
+  "OwnedItems": {
+    "SteelDagger": 1, "ThievesGuildCharm": 1, "LockpickSet": 2
+  },
+  "Role": "Thief",
+  "Relations": [
+    {"Target": "Vesper", "Favorability": 40},
+    {"Target": "RavenportSyndicate", "Favorability": 45},
+    {"Target": "SilverwoodCouncil", "Favorability": -40},
+    {"Target": "CaptainRook", "Favorability": 40},
+    {"Target": "DariusBlack", "Favorability": -15},
+    {"Target": "NyxShadowmere", "Favorability": 30}
+  ],
+  "NPCLog": []
+}
+UrgathBonebreaker: {
+  "Name": "UrgathBonebreaker",
+  "NamePossessive": "Urgath Bonebreaker's",
+  "Species": "Orc",
+  "HomeLocation": "Embermaw",
+  "CurrentLocation": "Embermaw",
+  "Faction": "EmbermawClan",
+  "OwnedItems": {
+    "IronSword": 1, "TrollFat": 3, "Rations": 5
+  },
+  "Role": "Mercenary",
+  "Relations": [
+    {"Target": "Vesper", "Favorability": -20},
+    {"Target": "EmbermawClan", "Favorability": 50},
+    {"Target": "RavenportSyndicate", "Favorability": -50},
+    {"Target": "RaskulGnarltooth", "Favorability": 35},
+    {"Target": "GrummokSkullcrusher", "Favorability": 40},
+    {"Target": "ThaliaIronfoot", "Favorability": 25}
+  ],
+  "NPCLog": []
+}
+MiloProudfoot: {
+  "Name": "MiloProudfoot",
+  "NamePossessive": "Milo Proudfoot's",
+  "Species": "Halfling",
+  "HomeLocation": "VerdantGlade",
+  "CurrentLocation": "Silverwood",
+  "Faction": "SilverwoodCouncil",
+  "OwnedItems": {
+    "Rations": 10, "HealthPotion": 2, "FishingRod": 1
+  },
+  "Role": "Innkeeper",
+  "Relations": [
+    {"Target": "Vesper", "Favorability": 30},
+    {"Target": "SilverwoodCouncil", "Favorability": 25},
+    {"Target": "RavenportSyndicate", "Favorability": -15},
+    {"Target": "LilyRosewater", "Favorability": 35},
+    {"Target": "FinnianSwift", "Favorability": 20},
+    {"Target": "HildaBarleybrew", "Favorability": -10}
+  ],
+  "NPCLog": []
+}
+SszikVess: {
+  "Name": "SszikVess",
+  "NamePossessive": "Sszik Vess's",
+  "Species": "Lizardfolk",
+  "HomeLocation": "Dreadmarsh",
+  "CurrentLocation": "Dreadmarsh",
+  "Faction": "EmbermawClan",
+  "OwnedItems": {
+    "ObsidianArrow": 10, "GoblinEar": 5, "Emberbloom": 3
+  },
+  "Role": "Hunter",
+  "Relations": [
+    {"Target": "Vesper", "Favorability": -5},
+    {"Target": "EmbermawClan", "Favorability": 30},
+    {"Target": "SilverwoodCouncil", "Favorability": -20},
+    {"Target": "UrgathBonebreaker", "Favorability": 20},
+    {"Target": "YgritteFrostbane", "Favorability": 25},
+    {"Target": "EldrinOakenshield", "Favorability": -15}
+  ],
+  "NPCLog": []
+}
+BrotherAlaric: {
+  "Name": "BrotherAlaric",
+  "NamePossessive": "Brother Alaric's",
+  "Species": "Human",
+  "HomeLocation": "Silverwood",
+  "CurrentLocation": "Silverwood",
+  "Faction": "SilverwoodCouncil",
+  "OwnedItems": {
+    "HealthPotion": 5, "SpellScrollLight": 1, "SilverRing": 1
+  },
+  "Role": "Priest",
+  "Relations": [
+    {"Target": "Vesper", "Favorability": 20},
+    {"Target": "SilverwoodCouncil", "Favorability": 40},
+    {"Target": "OrderOfTheSpire", "Favorability": 15},
+    {"Target": "KaelenSilverwood", "Favorability": 20},
+    {"Target": "AldricTrueblade", "Favorability": 35},
+    {"Target": "TiberiusGrimm", "Favorability": -10}
+  ],
+  "NPCLog": []
+}
+MadamVivienne: {
+  "Name": "MadamVivienne",
+  "NamePossessive": "Madam Vivienne's",
+  "Species": "Human",
+  "HomeLocation": "TheSpire",
+  "CurrentLocation": "TheSpire",
+  "Faction": "OrderOfTheSpire",
+  "OwnedItems": {
+    "EnchantedStaff": 1, "CrystalShard": 5, "ManaElixir": 4, "FrostMirror": 1
+  },
+  "Role": "Wizard",
+  "Relations": [
+    {"Target": "Vesper", "Favorability": 5},
+    {"Target": "OrderOfTheSpire", "Favorability": 50},
+    {"Target": "SilverwoodCouncil", "Favorability": 10},
+    {"Target": "ValeriusCorvus", "Favorability": 30},
+    {"Target": "ElaraMoonshadow", "Favorability": -5},
+    {"Target": "CaptainRook", "Favorability": -25}
+  ],
+  "NPCLog": []
+}
+OrinSteelhand: {
+  "Name": "OrinSteelhand",
+  "NamePossessive": "Orin Steelhand's",
+  "Species": "Dwarf",
+  "HomeLocation": "Ironhold",
+  "CurrentLocation": "Ironhold",
+  "Faction": "IronholdConglomerate",
+  "OwnedItems": {
+    "SturdyShield": 1, "IronSword": 1, "IronOre": 20
+  },
+  "Role": "GuardCaptain",
+  "Relations": [
+    {"Target": "Vesper", "Favorability": -15},
+    {"Target": "IronholdConglomerate", "Favorability": 50},
+    {"Target": "EmbermawClan", "Favorability": 20},
+    {"Target": "ThaliaIronfoot", "Favorability": 20},
+    {"Target": "GornHammerfall", "Favorability": 40},
+    {"Target": "DariusBlack", "Favorability": -35}
+  ],
+  "NPCLog": []
+}
+LilyRosewater: {
+  "Name": "LilyRosewater",
+  "NamePossessive": "Lily Rosewater's",
+  "Species": "Halfling",
+  "HomeLocation": "VerdantGlade",
+  "CurrentLocation": "VerdantGlade",
+  "Faction": "SilverwoodCouncil",
+  "OwnedItems": {
+    "GhostOrchid": 2, "HealthPotion": 3, "Rations": 8
+  },
+  "Role": "Apothecary",
+  "Relations": [
+    {"Target": "Vesper", "Favorability": 25},
+    {"Target": "SilverwoodCouncil", "Favorability": 20},
+    {"Target": "OrderOfTheSpire", "Favorability": -5},
+    {"Target": "MiloProudfoot", "Favorability": 35},
+    {"Target": "PennyHoneytongue", "Favorability": 20},
+    {"Target": "JasperWindleaf", "Favorability": -5}
+  ],
+  "NPCLog": []
+}
+DariusBlack: {
+  "Name": "DariusBlack",
+  "NamePossessive": "Darius Black's",
+  "Species": "Human",
+  "HomeLocation": "Ravenport",
+  "CurrentLocation": "Ravenport",
+  "Faction": "RavenportSyndicate",
+  "OwnedItems": {
+    "SteelDagger": 1, "LockpickSet": 1, "BlackPearl": 3
+  },
+  "Role": "Spy",
+  "Relations": [
+    {"Target": "Vesper", "Favorability": 45},
+    {"Target": "RavenportSyndicate", "Favorability": 35},
+    {"Target": "IronholdConglomerate", "Favorability": -25},
+    {"Target": "SeraphinaVex", "Favorability": -15},
+    {"Target": "MorganaDreadveil", "Favorability": 30},
+    {"Target": "OrinSteelhand", "Favorability": -35}
+  ],
+  "NPCLog": []
+}
+YgritteFrostbane: {
+  "Name": "YgritteFrostbane",
+  "NamePossessive": "Ygritte Frostbane's",
+  "Species": "Human",
+  "HomeLocation": "FrostfangPeak",
+  "CurrentLocation": "FrostfangPeak",
+  "Faction": "EmbermawClan",
+  "OwnedItems": {
+    "FrostMirror": 1, "CrystalShard": 3, "Rations": 4
+  },
+  "Role": "Hunter",
+  "Relations": [
+    {"Target": "Vesper", "Favorability": -35},
+    {"Target": "EmbermawClan", "Favorability": 40},
+    {"Target": "SilverwoodCouncil", "Favorability": -30},
+    {"Target": "SszikVess", "Favorability": 25},
+    {"Target": "VanyaStormrider", "Favorability": -20},
+    {"Target": "GrummokSkullcrusher", "Favorability": 20}
+  ],
+  "NPCLog": []
+}
+PercivalRustbucket: {
+  "Name": "PercivalRustbucket",
+  "NamePossessive": "Percival Rustbucket's",
+  "Species": "Gnome",
+  "HomeLocation": "TheSpire",
+  "CurrentLocation": "TheSpire",
+  "Faction": "OrderOfTheSpire",
+  "OwnedItems": {
+    "GrapplingHook": 1, "LockpickSet": 1, "FireSalt": 4, "ManaElixir": 1
+  },
+  "Role": "Alchemist",
+  "Relations": [
+    {"Target": "Vesper", "Favorability": 10},
+    {"Target": "OrderOfTheSpire", "Favorability": 30},
+    {"Target": "IronholdConglomerate", "Favorability": -10},
+    {"Target": "FizzwickTinkertop", "Favorability": 35},
+    {"Target": "OpalStardust", "Favorability": 25},
+    {"Target": "GrizzleGearspark", "Favorability": 5}
+  ],
+  "NPCLog": []
+}
+NyxShadowmere: {
+  "Name": "NyxShadowmere",
+  "NamePossessive": "Nyx Shadowmere's",
+  "Species": "Fae",
+  "HomeLocation": "Ravenport",
+  "CurrentLocation": "Dreadmarsh",
+  "Faction": "RavenportSyndicate",
+  "OwnedItems": {
+    "SteelDagger": 1, "ThievesGuildCharm": 1, "GhostOrchid": 2
+  },
+  "Role": "Thief",
+  "Relations": [
+    {"Target": "Vesper", "Favorability": 35},
+    {"Target": "RavenportSyndicate", "Favorability": 40},
+    {"Target": "SilverwoodCouncil", "Favorability": -45},
+    {"Target": "SeraphinaVex", "Favorability": 30},
+    {"Target": "SableFell", "Favorability": 40},
+    {"Target": "ElaraMoonshadow", "Favorability": -50}
+  ],
+  "NPCLog": []
+}
+GornHammerfall: {
+  "Name": "GornHammerfall",
+  "NamePossessive": "Gorn Hammerfall's",
+  "Species": "Dwarf",
+  "HomeLocation": "Ironhold",
+  "CurrentLocation": "Ironhold",
+  "Faction": "IronholdConglomerate",
+  "OwnedItems": {
+    "MiningPick": 1, "IronOre": 25, "AncientCoin": 100
+  },
+  "Role": "Miner",
+  "Relations": [
+    {"Target": "Vesper", "Favorability": -5},
+    {"Target": "IronholdConglomerate", "Favorability": 45},
+    {"Target": "EmbermawClan", "Favorability": 10},
+    {"Target": "BorinCoppervein", "Favorability": 40},
+    {"Target": "OrinSteelhand", "Favorability": 40},
+    {"Target": "RoricBoulderback", "Favorability": 35}
+  ],
+  "NPCLog": []
+}
+FizzwickTinkertop: {
+  "Name": "FizzwickTinkertop",
+  "NamePossessive": "Fizzwick Tinkertop's",
+  "Species": "Gnome",
+  "HomeLocation": "Ironhold",
+  "CurrentLocation": "Ironhold",
+  "Faction": "IronholdConglomerate",
+  "OwnedItems": {
+    "GrapplingHook": 2, "FireSalt": 6, "LockpickSet": 1
+  },
+  "Role": "Merchant",
+  "Relations": [
+    {"Target": "Vesper", "Favorability": 10},
+    {"Target": "IronholdConglomerate", "Favorability": 25},
+    {"Target": "OrderOfTheSpire", "Favorability": 5},
+    {"Target": "GrizzleGearspark", "Favorability": 25},
+    {"Target": "PercivalRustbucket", "Favorability": 35},
+    {"Target": "PennyHoneytongue", "Favorability": -15}
+  ],
+  "NPCLog": []
+}
+SeleneStarweaver: {
+  "Name": "SeleneStarweaver",
+  "NamePossessive": "Selene Starweaver's",
+  "Species": "Elf",
+  "HomeLocation": "Silverwood",
+  "CurrentLocation": "AzureCoast",
+  "Faction": "SilverwoodCouncil",
+  "OwnedItems": {
+    "EnchantedStaff": 1, "CrystalShard": 4, "SpellScrollLight": 2
+  },
+  "Role": "Wizard",
+  "Relations": [
+    {"Target": "Vesper", "Favorability": 15},
+    {"Target": "SilverwoodCouncil", "Favorability": 40},
+    {"Target": "OrderOfTheSpire", "Favorability": 15},
+    {"Target": "ElaraMoonshadow", "Favorability": 30},
+    {"Target": "ElysiaDawnseeker", "Favorability": 35},
+    {"Target": "MadamVivienne", "Favorability": -10}
+  ],
+  "NPCLog": []
+}
+BartholomewReed: {
+  "Name": "BartholomewReed",
+  "NamePossessive": "Bartholomew Reed's",
+  "Species": "Human",
+  "HomeLocation": "Ravenport",
+  "CurrentLocation": "Ravenport",
+  "Faction": "RavenportSyndicate",
+  "OwnedItems": {
+    "FishingRod": 1, "ShipManifest": 1, "BlackPearl": 1
+  },
+  "Role": "ShipCaptain",
+  "Relations": [
+    {"Target": "Vesper", "Favorability": 20},
+    {"Target": "RavenportSyndicate", "Favorability": 35},
+    {"Target": "SilverwoodCouncil", "Favorability": -20},
+    {"Target": "CaptainRook", "Favorability": 25},
+    {"Target": "QuinnSilverton", "Favorability": 30},
+    {"Target": "CyrusVance", "Favorability": -15}
+  ],
+  "NPCLog": []
+}
+RaskulGnarltooth: {
+  "Name": "RaskulGnarltooth",
+  "NamePossessive": "Raskul Gnarltooth's",
+  "Species": "Goblin",
+  "HomeLocation": "Embermaw",
+  "CurrentLocation": "Embermaw",
+  "Faction": "EmbermawClan",
+  "OwnedItems": {
+    "GoblinEar": 10, "ObsidianArrow": 5, "TrollFat": 2
+  },
+  "Role": "Hunter",
+  "Relations": [
+    {"Target": "Vesper", "Favorability": -25},
+    {"Target": "EmbermawClan", "Favorability": 40},
+    {"Target": "RavenportSyndicate", "Favorability": -45},
+    {"Target": "UrgathBonebreaker", "Favorability": 35},
+    {"Target": "GrobnikSneakwhistle", "Favorability": 30},
+    {"Target": "DariusBlack", "Favorability": -50}
+  ],
+  "NPCLog": []
+}
+MorganaDreadveil: {
+  "Name": "MorganaDreadveil",
+  "NamePossessive": "Morgana Dreadveil's",
+  "Species": "Human",
+  "HomeLocation": "Ravenport",
+  "CurrentLocation": "Ravenport",
+  "Faction": "RavenportSyndicate",
+  "OwnedItems": {
+    "SteelDagger": 1, "ThievesGuildCharm": 1, "BlackPearl": 2, "SilverRing": 1
+  },
+  "Role": "Spy",
+  "Relations": [
+    {"Target": "Vesper", "Favorability": 40},
+    {"Target": "RavenportSyndicate", "Favorability": 45},
+    {"Target": "SilverwoodCouncil", "Favorability": -45},
+    {"Target": "DariusBlack", "Favorability": 30},
+    {"Target": "Bell</t>
+  </si>
+  <si>
+    <t>## ENUM DATA
+{
+  "Types": {
+    "ItemTypes": ["Weapon", "Armor", "Potion", "Ingredient", "Key", "Artifact", "Currency", "Shield", "Tool", "Food"],
+    "QuestTypes": ["AttackThreateningEntities", "RecoverStolenItem", "GuardEntity", "AttackEnemy", "StealStuff", "KillEnemies"],
+    "EventTypes": ["Ambush", "Discovery", "Betrayal", "Alliance", "TradeRouteOpened", "ResourceDepleted", "Theft", "Rescue"],
+    "RelationshipLevels": {"Sworn Enemy": -50, "Enemy": -30, "Hated": -15, "Disliked": -5, "Neutral": 0, "Friendly": 5, "Friend": 15, "Ally": 30, "Sworn Ally": 50}
+  },
+  "Lists": {
+    "Species": ["Human", "Elf", "Dwarf", "Orc", "Halfling", "Lizardfolk"],
+    "Roles": ["Innkeeper", "Blacksmith", "Merchant", "GuardCaptain", "Apothecary", "Thief", "Wizard", "Ranger", "Bard", "Priest", "Alchemist", "Farmer", "Fisherman", "Hunter", "Miner", "Scholar", "Spy", "BountyHunter", "Mayor", "Stablemaster"],
+    "Locations": ["Stonehaven", "Ravenwood", "Ironpeak", "Shadowmere", "SunkissedFields", "TheWarrens", "HighCouncilChamber", "CrimsonBadlands", "WhisperingCaverns", "PortFrost"],
+    "Factions": ["TheIronGuard", "CircleOfWhispers", "MerchantsGuild", "ClanStonefist", "CrimsonOutriders"],
+    "Enemies": ["Wolf", "Bandit", "Skeleton", "Goblin", "Spider", "Troll", "Wraith", "OrcMarauder", "CaveBat", "Slime", "Harpy", "Gnoll", "Ogre", "Cultist", "Zombie", "GiantRat", "Elemental", "Assassin", "CorruptedElf", "Drake"],
+    "Items": ["IronSword", "LeatherArmor", "HealthPotion", "Nightshade", "RustyKey", "ElvenAmulet", "GoldCoin", "IronDagger", "SteelShield", "ManaPotion", "Bread", "Lockpick", "FishingRod", "WolfPelt", "IronOre", "MagesStaff", "ThievesGuildMissive", "DwarvenAle", "RubyGem", "AncientScroll", "GoblinEar", "BanditMask", "WraithDust", "TrollFat", "DrakeScale"],
+    "NPCs": ["Eldrin", "Thrain", "Lyra", "Gromm", "Milo", "Sera", "Borris", "Elara", "Kaelen", "Bram", "Nyx", "Orin", "Tessa", "Fizzwick", "Grizzle", "Valeria", "Cyrus", "Mira", "Roric", "Lilith", "Percival", "Isolde", "Fenris", "Willow", "Bronn", "Kira", "Magnus", "Reyna", "Theron", "Seraphina", "Zephyr", "Corvus", "Anya", "Dorian", "Gwen", "Jasper", "Selene", "Garrick", "Elowen", "Thorne", "Rosie", "Balthazar", "Morgana", "Grunt", "Felix", "Rowan", "Brynn", "Alistair", "Vex", "Pip", "Glimmer", "Zara", "Hilda"],
+    "Player": ["TheWanderer"]
+  }
+}
+;
+### ITEM DATA
+IronSword: { 
+  "Type": "Weapon", 
+  "Name": "Iron Sword", 
+  "NameSingular": "Iron Sword", 
+  "NamePlural": "Iron Swords",
+  "NamePossessiveSingular": "Iron Sword's",
+  "NamePossessivePlural": "Iron Swords'",
+  "IndefiniteArticle": "an",
+  "IndefiniteArticleCaps": "An"
+}
+LeatherArmor: { 
+  "Type": "Armor", 
+  "Name": "Leather Armor", 
+  "NameSingular": "Leather Armor", 
+  "NamePlural": "Leather Armors",
+  "NamePossessiveSingular": "Leather Armor's",
+  "NamePossessivePlural": "Leather Armors'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+HealthPotion: { 
+  "Type": "Potion", 
+  "Name": "Health Potion", 
+  "NameSingular": "Health Potion", 
+  "NamePlural": "Health Potions",
+  "NamePossessiveSingular": "Health Potion's",
+  "NamePossessivePlural": "Health Potions'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+Nightshade: { 
+  "Type": "Ingredient", 
+  "Name": "Nightshade", 
+  "NameSingular": "Nightshade", 
+  "NamePlural": "Nightshades",
+  "NamePossessiveSingular": "Nightshade's",
+  "NamePossessivePlural": "Nightshades'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+RustyKey: { 
+  "Type": "Key", 
+  "Name": "Rusty Key", 
+  "NameSingular": "Rusty Key", 
+  "NamePlural": "Rusty Keys",
+  "NamePossessiveSingular": "Rusty Key's",
+  "NamePossessivePlural": "Rusty Keys'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+ElvenAmulet: { 
+  "Type": "Artifact", 
+  "Name": "Elven Amulet", 
+  "NameSingular": "Elven Amulet", 
+  "NamePlural": "Elven Amulets",
+  "NamePossessiveSingular": "Elven Amulet's",
+  "NamePossessivePlural": "Elven Amulets'",
+  "IndefiniteArticle": "an",
+  "IndefiniteArticleCaps": "An"
+}
+GoldCoin: { 
+  "Type": "Currency", 
+  "Name": "Gold Coin", 
+  "NameSingular": "Gold Coin", 
+  "NamePlural": "Gold Coins",
+  "NamePossessiveSingular": "Gold Coin's",
+  "NamePossessivePlural": "Gold Coins'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+IronDagger: { 
+  "Type": "Weapon", 
+  "Name": "Iron Dagger", 
+  "NameSingular": "Iron Dagger", 
+  "NamePlural": "Iron Daggers",
+  "NamePossessiveSingular": "Iron Dagger's",
+  "NamePossessivePlural": "Iron Daggers'",
+  "IndefiniteArticle": "an",
+  "IndefiniteArticleCaps": "An"
+}
+SteelShield: { 
+  "Type": "Shield", 
+  "Name": "Steel Shield", 
+  "NameSingular": "Steel Shield", 
+  "NamePlural": "Steel Shields",
+  "NamePossessiveSingular": "Steel Shield's",
+  "NamePossessivePlural": "Steel Shields'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+ManaPotion: { 
+  "Type": "Potion", 
+  "Name": "Mana Potion", 
+  "NameSingular": "Mana Potion", 
+  "NamePlural": "Mana Potions",
+  "NamePossessiveSingular": "Mana Potion's",
+  "NamePossessivePlural": "Mana Potions'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+Bread: { 
+  "Type": "Food", 
+  "Name": "Bread", 
+  "NameSingular": "Bread", 
+  "NamePlural": "Breads",
+  "NamePossessiveSingular": "Bread's",
+  "NamePossessivePlural": "Breads'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+Lockpick: { 
+  "Type": "Tool", 
+  "Name": "Lockpick", 
+  "NameSingular": "Lockpick", 
+  "NamePlural": "Lockpicks",
+  "NamePossessiveSingular": "Lockpick's",
+  "NamePossessivePlural": "Lockpicks'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+FishingRod: { 
+  "Type": "Tool", 
+  "Name": "Fishing Rod", 
+  "NameSingular": "Fishing Rod", 
+  "NamePlural": "Fishing Rods",
+  "NamePossessiveSingular": "Fishing Rod's",
+  "NamePossessivePlural": "Fishing Rods'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+WolfPelt: { 
+  "Type": "Ingredient", 
+  "Name": "Wolf Pelt", 
+  "NameSingular": "Wolf Pelt", 
+  "NamePlural": "Wolf Pelts",
+  "NamePossessiveSingular": "Wolf Pelt's",
+  "NamePossessivePlural": "Wolf Pelts'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+IronOre: { 
+  "Type": "Ingredient", 
+  "Name": "Iron Ore", 
+  "NameSingular": "Iron Ore", 
+  "NamePlural": "Iron Ores",
+  "NamePossessiveSingular": "Iron Ore's",
+  "NamePossessivePlural": "Iron Ores'",
+  "IndefiniteArticle": "an",
+  "IndefiniteArticleCaps": "An"
+}
+MagesStaff: { 
+  "Type": "Weapon", 
+  "Name": "Mage's Staff", 
+  "NameSingular": "Mage's Staff", 
+  "NamePlural": "Mage's Staves",
+  "NamePossessiveSingular": "Mage's Staff's",
+  "NamePossessivePlural": "Mage's Staves'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+ThievesGuildMissive: { 
+  "Type": "Key", 
+  "Name": "Thieves Guild Missive", 
+  "NameSingular": "Thieves Guild Missive", 
+  "NamePlural": "Thieves Guild Missives",
+  "NamePossessiveSingular": "Thieves Guild Missive's",
+  "NamePossessivePlural": "Thieves Guild Missives'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+DwarvenAle: { 
+  "Type": "Food", 
+  "Name": "Dwarven Ale", 
+  "NameSingular": "Dwarven Ale", 
+  "NamePlural": "Dwarven Ales",
+  "NamePossessiveSingular": "Dwarven Ale's",
+  "NamePossessivePlural": "Dwarven Ales'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+RubyGem: { 
+  "Type": "Currency", 
+  "Name": "Ruby Gem", 
+  "NameSingular": "Ruby Gem", 
+  "NamePlural": "Ruby Gems",
+  "NamePossessiveSingular": "Ruby Gem's",
+  "NamePossessivePlural": "Ruby Gems'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+AncientScroll: { 
+  "Type": "Artifact", 
+  "Name": "Ancient Scroll", 
+  "NameSingular": "Ancient Scroll", 
+  "NamePlural": "Ancient Scrolls",
+  "NamePossessiveSingular": "Ancient Scroll's",
+  "NamePossessivePlural": "Ancient Scrolls'",
+  "IndefiniteArticle": "an",
+  "IndefiniteArticleCaps": "An"
+}
+GoblinEar: { 
+  "Type": "Ingredient", 
+  "Name": "Goblin Ear", 
+  "NameSingular": "Goblin Ear", 
+  "NamePlural": "Goblin Ears",
+  "NamePossessiveSingular": "Goblin Ear's",
+  "NamePossessivePlural": "Goblin Ears'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+BanditMask: { 
+  "Type": "Armor", 
+  "Name": "Bandit Mask", 
+  "NameSingular": "Bandit Mask", 
+  "NamePlural": "Bandit Masks",
+  "NamePossessiveSingular": "Bandit Mask's",
+  "NamePossessivePlural": "Bandit Masks'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+WraithDust: { 
+  "Type": "Ingredient", 
+  "Name": "Wraith Dust", 
+  "NameSingular": "Wraith Dust", 
+  "NamePlural": "Wraith Dusts",
+  "NamePossessiveSingular": "Wraith Dust's",
+  "NamePossessivePlural": "Wraith Dusts'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+TrollFat: { 
+  "Type": "Ingredient", 
+  "Name": "Troll Fat", 
+  "NameSingular": "Troll Fat", 
+  "NamePlural": "Troll Fats",
+  "NamePossessiveSingular": "Troll Fat's",
+  "NamePossessivePlural": "Troll Fats'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+DrakeScale: { 
+  "Type": "Ingredient", 
+  "Name": "Drake Scale", 
+  "NameSingular": "Drake Scale", 
+  "NamePlural": "Drake Scales",
+  "NamePossessiveSingular": "Drake Scale's",
+  "NamePossessivePlural": "Drake Scales'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+;
+## GAME STATE DATA
+### FACTION DATA
+TheIronGuard: {
+  "Name": "The Iron Guard", 
+  "NameDefinitive": "the Iron Guard",
+  "NameDefinitiveCaps": "The Iron Guard",
+  "NamePossessive": "The Iron Guard's",
+  "NameDefinitivePossessive": "the Iron Guard's",
+  "NameDefinitivePossessiveCaps": "The Iron Guard's",
+  "DefaultLocation": "Stonehaven",
+  "Relations": [
+    {"Target": "TheWanderer", "Favorability": 15},
+    {"Target": "CircleOfWhispers", "Favorability": -20},
+    {"Target": "MerchantsGuild", "Favorability": 10},
+    {"Target": "ClanStonefist", "Favorability": 25},
+    {"Target": "CrimsonOutriders", "Favorability": -40}
+  ],
+  "Members": ["Borris", "Valeria", "Alistair", "Brynn", "Gwen", "Reyna", "Orin", "Hilda"],
+  "Treasury": {
+    "IronSword": 15,
+    "SteelShield": 10,
+    "LeatherArmor": 20,
+    "GoldCoin": 5000,
+    "HealthPotion": 50,
+    "IronOre": 100
+  },
+  "FactionLog": []
+}
+CircleOfWhispers: {
+  "Name": "The Circle of Whispers", 
+  "NameDefinitive": "the Circle of Whispers",
+  "NameDefinitiveCaps": "The Circle of Whispers",
+  "NamePossessive": "The Circle of Whispers'",
+  "NameDefinitivePossessive": "the Circle of Whispers'",
+  "NameDefinitivePossessiveCaps": "The Circle of Whispers'",
+  "DefaultLocation": "Shadowmere",
+  "Relations": [
+    {"Target": "TheWanderer", "Favorability": 5},
+    {"Target": "TheIronGuard", "Favorability": -20},
+    {"Target": "MerchantsGuild", "Favorability": 5},
+    {"Target": "ClanStonefist", "Favorability": -5},
+    {"Target": "CrimsonOutriders", "Favorability": 30}
+  ],
+  "Members": ["Nyx", "Cyrus", "Lilith", "Corvus", "Vex", "Seraphina", "Zephyr", "Morgana"],
+  "Treasury": {
+    "IronDagger": 25,
+    "Lockpick": 50,
+    "Nightshade": 30,
+    "ThievesGuildMissive": 10,
+    "GoldCoin": 8000,
+    "ManaPotion": 20
+  },
+  "FactionLog": []
+}
+MerchantsGuild: {
+  "Name": "The Merchants Guild", 
+  "NameDefinitive": "the Merchants Guild",
+  "NameDefinitiveCaps": "The Merchants Guild",
+  "NamePossessive": "The Merchants Guild's",
+  "NameDefinitivePossessive": "the Merchants Guild's",
+  "NameDefinitivePossessiveCaps": "The Merchants Guild's",
+  "DefaultLocation": "PortFrost",
+  "Relations": [
+    {"Target": "TheWanderer", "Favorability": 10},
+    {"Target": "TheIronGuard", "Favorability": 10},
+    {"Target": "CircleOfWhispers", "Favorability": 5},
+    {"Target": "ClanStonefist", "Favorability": 15},
+    {"Target": "CrimsonOutriders", "Favorability": -10}
+  ],
+  "Members": ["Milo", "Tessa", "Percival", "Rosie", "Felix", "Anya", "Dorian", "Jasper"],
+  "Treasury": {
+    "GoldCoin": 25000,
+    "RubyGem": 15,
+    "Bread": 100,
+    "FishingRod": 10,
+    "WolfPelt": 40,
+    "DwarvenAle": 30
+  },
+  "FactionLog": []
+}
+ClanStonefist: {
+  "Name": "Clan Stonefist", 
+  "NameDefinitive": "Clan Stonefist",
+  "NameDefinitiveCaps": "Clan Stonefist",
+  "NamePossessive": "Clan Stonefist's",
+  "NameDefinitivePossessive": "Clan Stonefist's",
+  "NameDefinitivePossessiveCaps": "Clan Stonefist's",
+  "DefaultLocation": "Ironpeak",
+  "Relations": [
+    {"Target": "TheWanderer", "Favorability": 25},
+    {"Target": "TheIronGuard", "Favorability": 25},
+    {"Target": "CircleOfWhispers", "Favorability": -5},
+    {"Target": "MerchantsGuild", "Favorability": 15},
+    {"Target": "CrimsonOutriders", "Favorability": -15}
+  ],
+  "Members": ["Thrain", "Roric", "Magnus", "Hilda", "Bram", "Grizzle", "Fizzwick", "Bronn"],
+  "Treasury": {
+    "IronOre": 500,
+    "GoldCoin": 12000,
+    "DwarvenAle": 80,
+    "IronSword": 30,
+    "SteelShield": 25,
+    "RubyGem": 5
+  },
+  "FactionLog": []
+}
+CrimsonOutriders: {
+  "Name": "The Crimson Outriders", 
+  "NameDefinitive": "the Crimson Outriders",
+  "NameDefinitiveCaps": "The Crimson Outriders",
+  "NamePossessive": "The Crimson Outriders'",
+  "NameDefinitivePossessive": "the Crimson Outriders'",
+  "NameDefinitivePossessiveCaps": "The Crimson Outriders'",
+  "DefaultLocation": "CrimsonBadlands",
+  "Relations": [
+    {"Target": "TheWanderer", "Favorability": -30},
+    {"Target": "TheIronGuard", "Favorability": -40},
+    {"Target": "CircleOfWhispers", "Favorability": 30},
+    {"Target": "MerchantsGuild", "Favorability": -10},
+    {"Target": "ClanStonefist", "Favorability": -15}
+  ],
+  "Members": ["Gromm", "Kaelen", "Fenris", "Grunt", "Theron", "Zara", "Thorne", "Sera"],
+  "Treasury": {
+    "IronSword": 40,
+    "LeatherArmor": 35,
+    "BanditMask": 20,
+    "GoldCoin": 7000,
+    "HealthPotion": 15,
+    "WolfPelt": 50
+  },
+  "FactionLog": []
+}
+;
+### NPC DATA
+Eldrin: {
+  "Name": "Eldrin",
+  "NamePossessive": "Eldrin's",
+  "Species": "Elf",
+  "HomeLocation": "Ravenwood",
+  "CurrentLocation": "Ravenwood",
+  "Faction": null,
+  "OwnedItems": {
+    "ElvenAmulet": 1,
+    "ManaPotion": 3,
+    "AncientScroll": 2
+  },
+  "Role": "Wizard",
+  "Relations": [
+    {"Target": "TheWanderer", "Favorability": 20},
+    {"Target": "CircleOfWhispers", "Favorability": 10},
+    {"Target": "Lyra", "Favorability": 35},
+    {"Target": "Kaelen", "Favorability": -40},
+    {"Target": "Gromm", "Favorability": -25},
+    {"Target": "Seraphina", "Favorability": 15},
+    {"Target": "Corvus", "Favorability": -10}
+  ],
+  "NPCLog": []
+}
+Thrain: {
+  "Name": "Thrain",
+  "NamePossessive": "Thrain's",
+  "Species": "Dwarf",
+  "HomeLocation": "Ironpeak",
+  "CurrentLocation": "Ironpeak",
+  "Faction": "ClanStonefist",
+  "OwnedItems": {
+    "IronSword": 1,
+    "DwarvenAle": 5,
+    "RubyGem": 2
+  },
+  "Role": "Blacksmith",
+  "Relations": [
+    {"Target": "TheWanderer", "Favorability": 30},
+    {"Target": "ClanStonefist", "Favorability": 50},
+    {"Target": "TheIronGuard", "Favorability": 15},
+    {"Target": "Roric", "Favorability": 40},
+    {"Target": "Borris", "Favorability": 25},
+    {"Target": "Nyx", "Favorability": -20},
+    {"Target": "Gromm", "Favorability": -35}
+  ],
+  "NPCLog": []
+}
+Lyra: {
+  "Name": "Lyra",
+  "NamePossessive": "Lyra's",
+  "Species": "Elf",
+  "HomeLocation": "Ravenwood",
+  "CurrentLocation": "Stonehaven",
+  "Faction": null,
+  "OwnedItems": {
+    "HealthPotion": 5,
+    "Nightshade": 3,
+    "Bread": 2
+  },
+  "Role": "Apothecary",
+  "Relations": [
+    {"Target": "TheWanderer", "Favorability": 25},
+    {"Target": "TheIronGuard", "Favorability": 10},
+    {"Target": "Eldrin", "Favorability": 35},
+    {"Target": "Valeria", "Favorability": 20},
+    {"Target": "Cyrus", "Favorability": -15},
+    {"Target": "Fenris", "Favorability": -30}
+  ],
+  "NPCLog": []
+}
+Gromm: {
+  "Name": "Gromm",
+  "NamePossessive": "Gromm's",
+  "Species": "Orc",
+  "HomeLocation": "CrimsonBadlands",
+  "CurrentLocation": "CrimsonBadlands",
+  "Faction": "CrimsonOutriders",
+  "OwnedItems": {
+    "IronSword": 1,
+    "BanditMask": 1,
+    "HealthPotion": 2
+  },
+  "Role": "BountyHunter",
+  "Relations": [
+    {"Target": "TheWanderer", "Favorability": -45},
+    {"Target": "CrimsonOutriders", "Favorability": 45},
+    {"Target": "TheIronGuard", "Favorability": -50},
+    {"Target": "Kaelen", "Favorability": 40},
+    {"Target": "Thrain", "Favorability": -35},
+    {"Target": "Eldrin", "Favorability": -30},
+    {"Target": "Borris", "Favorability": -50}
+  ],
+  "NPCLog": []
+}
+Milo: {
+  "Name": "Milo",
+  "NamePossessive": "Milo's",
+  "Species": "Halfling",
+  "HomeLocation": "SunkissedFields",
+  "CurrentLocation": "PortFrost",
+  "Faction": "MerchantsGuild",
+  "OwnedItems": {
+    "GoldCoin": 50,
+    "Bread": 10,
+    "FishingRod": 1
+  },
+  "Role": "Merchant",
+  "Relations": [
+    {"Target": "TheWanderer", "Favorability": 15},
+    {"Target": "MerchantsGuild", "Favorability": 40},
+    {"Target": "Tessa", "Favorability": 30},
+    {"Target": "Percival", "Favorability": 25},
+    {"Target": "Vex", "Favorability": -20},
+    {"Target": "Nyx", "Favorability": -15}
+  ],
+  "NPCLog": []
+}
+Sera: {
+  "Name": "Sera",
+  "NamePossessive": "Sera's",
+  "Species": "Human",
+  "HomeLocation": "CrimsonBadlands",
+  "CurrentLocation": "Shadowmere",
+  "Faction": "CrimsonOutriders",
+  "OwnedItems": {
+    "IronDagger": 2,
+    "Lockpick": 5,
+    "ThievesGuildMissive": 1
+  },
+  "Role": "Spy",
+  "Relations": [
+    {"Target": "TheWanderer", "Favorability": 5},
+    {"Target": "CrimsonOutriders", "Favorability": 35},
+    {"Target": "CircleOfWhispers", "Favorability": 20},
+    {"Target": "Lilith", "Favorability": 30},
+    {"Target": "Cyrus", "Favorability": 25},
+    {"Target": "Valeria", "Favorability": -30},
+    {"Target": "Alistair", "Favorability": -25}
+  ],
+  "NPCLog": []
+}
+Borris: {
+  "Name": "Borris",
+  "NamePossessive": "Borris'",
+  "Species": "Human",
+  "HomeLocation": "Stonehaven",
+  "CurrentLocation": "Stonehaven",
+  "Faction": "TheIronGuard",
+  "OwnedItems": {
+    "SteelShield": 1,
+    "IronSword": 1,
+    "LeatherArmor": 1
+  },
+  "Role": "GuardCaptain",
+  "Relations": [
+    {"Target": "TheWanderer", "Favorability": 20},
+    {"Target": "TheIronGuard", "Favorability": 50},
+    {"Target": "Valeria", "Favorability": 45},
+    {"Target": "Alistair", "Favorability": 40},
+    {"Target": "Gromm", "Favorability": -50},
+    {"Target": "Kaelen", "Favorability": -45},
+    {"Target": "Nyx", "Favorability": -20}
+  ],
+  "NPCLog": []
+}
+Elara: {
+  "Name": "Elara",
+  "NamePossessive": "Elara's",
+  "Species": "Elf",
+  "HomeLocation": "Ravenwood",
+  "CurrentLocation": "HighCouncilChamber",
+  "Faction": null,
+  "OwnedItems": {
+    "MagesStaff": 1,
+    "ManaPotion": 5,
+    "AncientScroll": 3
+  },
+  "Role": "Scholar",
+  "Relations": [
+    {"Target": "TheWanderer", "Favorability": 10},
+    {"Target": "CircleOfWhispers", "Favorability": 5},
+    {"Target": "Eldrin", "Favorability": 20},
+    {"Target": "Seraphina", "Favorability": 15},
+    {"Target": "Theron", "Favorability": -15}
+  ],
+  "NPCLog": []
+}
+Kaelen: {
+  "Name": "Kaelen",
+  "NamePossessive": "Kaelen's",
+  "Species": "Lizardfolk",
+  "HomeLocation": "CrimsonBadlands",
+  "CurrentLocation": "CrimsonBadlands",
+  "Faction": "CrimsonOutriders",
+  "OwnedItems": {
+    "IronSword": 1,
+    "WolfPelt": 3,
+    "TrollFat": 2
+  },
+  "Role": "Hunter",
+  "Relations": [
+    {"Target": "TheWanderer", "Favorability": -40},
+    {"Target": "CrimsonOutriders", "Favorability": 40},
+    {"Target": "Gromm", "Favorability": 40},
+    {"Target": "Fenris", "Favorability": 35},
+    {"Target": "Borris", "Favorability": -45},
+    {"Target": "Eldrin", "Favorability": -40},
+    {"Target": "Valeria", "Favorability": -35}
+  ],
+  "NPCLog": []
+}
+Bram: {
+  "Name": "Bram",
+  "NamePossessive": "Bram's",
+  "Species": "Dwarf",
+  "HomeLocation": "Ironpeak",
+  "CurrentLocation": "Ironpeak",
+  "Faction": "ClanStonefist",
+  "OwnedItems": {
+    "IronOre": 10,
+    "DwarvenAle": 3,
+    "GoldCoin": 25
+  },
+  "Role": "Miner",
+  "Relations": [
+    {"Target": "TheWanderer", "Favorability": 20},
+    {"Target": "ClanStonefist", "Favorability": 45},
+    {"Target": "Thrain", "Favorability": 35},
+    {"Target": "Roric", "Favorability": 30},
+    {"Target": "Nyx", "Favorability": -10}
+  ],
+  "NPCLog": []
+}
+Nyx: {
+  "Name": "Nyx",
+  "NamePossessive": "Nyx's",
+  "Species": "Halfling",
+  "HomeLocation": "Shadowmere",
+  "CurrentLocation": "Shadowmere",
+  "Faction": "CircleOfWhispers",
+  "OwnedItems": {
+    "IronDagger": 2,
+    "Lockpick": 10,
+    "Nightshade": 5
+  },
+  "Role": "Thief",
+  "Relations": [
+    {"Target": "TheWanderer", "Favorability": -5},
+    {"Target": "CircleOfWhispers", "Favorability": 45},
+    {"Target": "Cyrus", "Favorability": 35},
+    {"Target": "Vex", "Favorability": 40},
+    {"Target": "Borris", "Favorability": -30},
+    {"Target": "Valeria", "Favorability": -25},
+    {"Target": "Thrain", "Favorability": -20}
+  ],
+  "NPCLog": []
+}
+Orin: {
+  "Name": "Orin",
+  "NamePossessive": "Orin's",
+  "Species": "Human",
+  "HomeLocation": "Stonehaven",
+  "CurrentLocation": "Stonehaven",
+  "Faction": "TheIronGuard",
+  "OwnedItems": {
+    "IronSword": 1,
+    "LeatherArmor": 1,
+    "HealthPotion": 2
+  },
+  "Role": "GuardCaptain",
+  "Relations": [
+    {"Target": "TheWanderer", "Favorability": 15},
+    {"Target": "TheIronGuard", "Favorability": 40},
+    {"Target": "Borris", "Favorability": 35},
+    {"Target": "Alistair", "Favorability": 30},
+    {"Target": "Gromm", "Favorability": -40}
+  ],
+  "NPCLog": []
+}
+Tessa: {
+  "Name": "Tessa",
+  "NamePossessive": "Tessa's",
+  "Species": "Human",
+  "HomeLocation": "PortFrost",
+  "CurrentLocation": "PortFrost",
+  "Faction": "MerchantsGuild",
+  "OwnedItems": {
+    "GoldCoin": 100,
+    "RubyGem": 1,
+    "FishingRod": 1
+  },
+  "Role": "Merchant",
+  "Relations": [
+    {"Target": "TheWanderer", "Favorability": 10},
+    {"Target": "MerchantsGuild", "Favorability": 35},
+    {"Target": "Milo", "Favorability": 30},
+    {"Target": "Percival", "Favorability": 25},
+    {"Target": "Fenris", "Favorability": -15}
+  ],
+  "NPCLog": []
+}
+Fizzwick: {
+  "Name": "Fizzwick",
+  "NamePossessive": "Fizzwick's",
+  "Species": "Halfling",
+  "HomeLocation": "Ironpeak",
+  "CurrentLocation": "Ironpeak",
+  "Faction": "ClanStonefist",
+  "OwnedItems": {
+    "DwarvenAle": 10,
+    "Bread": 5,
+    "GoldCoin": 15
+  },
+  "Role": "Innkeeper",
+  "Relations": [
+    {"Target": "TheWanderer", "Favorability": 30},
+    {"Target": "ClanStonefist", "Favorability": 30},
+    {"Target": "Thrain", "Favorability": 25},
+    {"Target": "Bram", "Favorability": 20},
+    {"Target": "Vex", "Favorability": -10}
+  ],
+  "NPCLog": []
+}
+Grizzle: {
+  "Name": "Grizzle",
+  "NamePossessive": "Grizzle's",
+  "Species": "Dwarf",
+  "HomeLocation": "Ironpeak",
+  "CurrentLocation": "Ironpeak",
+  "Faction": "ClanStonefist",
+  "OwnedItems": {
+    "IronOre": 15,
+    "IronSword": 1,
+    "HealthPotion": 1
+  },
+  "Role": "Miner",
+  "Relations": [
+    {"Target": "TheWanderer", "Favorability": 15},
+    {"Target": "ClanStonefist", "Favorability": 40},
+    {"Target": "Bram", "Favorability": 35},
+    {"Target": "Thrain", "Favorability": 20},
+    {"Target": "Cyrus", "Favorability": -5}
+  ],
+  "NPCLog": []
+}
+Valeria: {
+  "Name": "Valeria",
+  "NamePossessive": "Valeria's",
+  "Species": "Human",
+  "HomeLocation": "Stonehaven",
+  "CurrentLocation": "Stonehaven",
+  "Faction": "TheIronGuard",
+  "OwnedItems": {
+    "SteelShield": 1,
+    "IronSword": 1,
+    "HealthPotion": 3
+  },
+  "Role": "GuardCaptain",
+  "Relations": [
+    {"Target": "TheWanderer", "Favorability": 25},
+    {"Target": "TheIronGuard", "Favorability": 50},
+    {"Target": "Borris", "Favorability": 45},
+    {"Target": "Alistair", "Favorability": 40},
+    {"Target": "Gromm", "Favorability": -50},
+    {"Target": "Kaelen", "Favorability": -45},
+    {"Target": "Nyx", "Favorability": -25}
+  ],
+  "NPCLog": []
+}
+Cyrus: {
+  "Name": "Cyrus",
+  "NamePossessive": "Cyrus'",
+  "Species": "Human",
+  "HomeLocation": "Shadowmere",
+  "CurrentLocation": "Shadowmere",
+  "Faction": "CircleOfWhispers",
+  "OwnedItems": {
+    "IronDagger": 1,
+    "Lockpick": 5,
+    "ThievesGuildMissive": 2
+  },
+  "Role": "Spy",
+  "Relations": [
+    {"Target": "TheWanderer", "Favorability": 0},
+    {"Target": "CircleOfWhispers", "Favorability": 40},
+    {"Target": "Nyx", "Favorability": 35},
+    {"Target": "Lilith", "Favorability": 30},
+    {"Target": "Borris", "Favorability": -35},
+    {"Target": "Valeria", "Favorability": -30},
+    {"Target": "Lyra", "Favorability": -15}
+  ],
+  "NPCLog": []
+}
+Mira: {
+  "Name": "Mira",
+  "NamePossessive": "Mira's",
+  "Species": "Elf",
+  "HomeLocation": "Ravenwood",
+  "CurrentLocation": "WhisperingCaverns",
+  "Faction": null,
+  "OwnedItems": {
+    "ManaPotion": 3,
+    "Nightshade": 5,
+    "AncientScroll": 1
+  },
+  "Role": "Alchemist",
+  "Relations": [
+    {"Target": "TheWanderer", "Favorability": 5},
+    {"Target": "CircleOfWhispers", "Favorability": 0},
+    {"Target": "Lyra", "Favorability": 15},
+    {"Target": "Eldrin", "Favorability": 10}
+  ],
+  "NPCLog": []
+}
+Roric: {
+  "Name": "Roric",
+  "NamePossessive": "Roric's",
+  "Species": "Dwarf",
+  "HomeLocation": "Ironpeak",
+  "CurrentLocation": "Ironpeak",
+  "Faction": "ClanStonefist",
+  "OwnedItems": {
+    "IronSword": 1,
+    "SteelShield": 1,
+    "DwarvenAle": 5
+  },
+  "Role": "Blacksmith",
+  "Relations": [
+    {"Target": "TheWanderer", "Favorability": 20},
+    {"Target": "ClanStonefist", "Favorability": 45},
+    {"Target": "Thrain", "Favorability": 40},
+    {"Target": "Bram", "Favorability": 30},
+    {"Target": "Gromm", "Favorability": -30}
+  ],
+  "NPCLog": []
+}
+Lilith: {
+  "Name": "Lilith",
+  "NamePossessive": "Lilith's",
+  "Species": "Lizardfolk",
+  "HomeLocation": "Shadowmere",
+  "CurrentLocation": "Shadowmere",
+  "Faction": "CircleOfWhispers",
+  "OwnedItems": {
+    "IronDagger": 2,
+    "Nightshade": 3,
+    "WraithDust": 1
+  },
+  "Role": "Assassin",
+  "Relations": [
+    {"Target": "TheWanderer", "Favorability": -10},
+    {"Target": "CircleOfWhispers", "Favorability": 35},
+    {"Target": "Nyx", "Favorability": 30},
+    {"Target": "Cyrus", "Favorability": 30},
+    {"Target": "Sera", "Favorability": 25},
+    {"Target": "Borris", "Favorability": -40},
+    {"Target": "Alistair", "Favorability": -35}
+  ],
+  "NPCLog": []
+}
+Percival: {
+  "Name": "Percival",
+  "NamePossessive": "Percival's",
+  "Species": "Human",
+  "HomeLocation": "PortFrost",
+  "CurrentLocation": "PortFrost",
+  "Faction": "MerchantsGuild",
+  "OwnedItems": {
+    "GoldCoin": 200,
+    "RubyGem": 3,
+    "WolfPelt": 5
+  },
+  "Role": "Merchant",
+  "Relations": [
+    {"Target": "TheWanderer", "Favorability": 5},
+    {"Target": "MerchantsGuild", "Favorability": 30},
+    {"Target": "Milo", "Favorability": 25},
+    {"Target": "Tessa", "Favorability": 25},
+    {"Target": "Fenris", "Favorability": -20}
+  ],
+  "NPCLog": []
+}
+Isolde: {
+  "Name": "Isolde",
+  "NamePossessive": "Isolde's",
+  "Species": "Elf",
+  "HomeLocation": "Ravenwood",
+  "CurrentLocation": "Ravenwood",
+  "Faction": null,
+  "OwnedItems": {
+    "ElvenAmulet": 1,
+    "ManaPotion": 2,
+    "HealthPotion": 3
+  },
+  "Role": "Priest",
+  "Relations": [
+    {"Target": "TheWanderer", "Favorability": 15},
+    {"Target": "Eldrin", "Favorability": 25},
+    {"Target": "Lyra", "Favorability": 20},
+    {"Target": "Theron", "Favorability": -10}
+  ],
+  "NPCLog": []
+}
+Fenris: {
+  "Name": "Fenris",
+  "NamePossessive": "Fenris'",
+  "Species": "Orc",
+  "HomeLocation": "CrimsonBadlands",
+  "CurrentLocation": "CrimsonBadlands",
+  "Faction": "CrimsonOutriders",
+  "OwnedItems": {
+    "IronSword": 1,
+    "WolfPelt": 4,
+    "BanditMask": 1
+  },
+  "Role": "Hunter",
+  "Relations": [
+    {"Target": "TheWanderer", "Favorability": -35},
+    {"Target": "CrimsonOutriders", "Favorability": 35},
+    {"Target": "Gromm", "Favorability": 30},
+    {"Target": "Kaelen", "Favorability": 35},
+    {"Target": "Valeria", "Favorability": -40},
+    {"Target": "Lyra", "Favorability": -30}
+  ],
+  "NPCLog": []
+}
+Willow: {
+  "Name": "Willow",
+  "NamePossessive": "Willow's",
+  "Species": "Halfling",
+  "HomeLocation": "SunkissedFields",
+  "CurrentLocation": "SunkissedFields",
+  "Faction": null,
+  "OwnedItems": {
+    "Bread": 10,
+    "FishingRod": 1,
+    "HealthPotion": 1
+  },
+  "Role": "Farmer",
+  "Relations": [
+    {"Target": "TheWanderer", "Favorability": 20},
+    {"Target": "MerchantsGuild", "Favorability": 15},
+    {"Target": "Milo", "Favorability": 20},
+    {"Target": "Rosie", "Favorability": 30}
+  ],
+  "NPCLog": []
+}
+Bronn: {
+  "Name": "Bronn",
+  "NamePossessive": "Bronn's",
+  "Species": "Dwarf",
+  "HomeLocation": "Ironpeak",
+  "CurrentLocation": "Stonehaven",
+  "Faction": "ClanStonefist",
+  "OwnedItems": {
+    "IronOre": 20,
+    "GoldCoin": 30,
+    "DwarvenAle": 2
+  },
+  "Role": "Miner",
+  "Relations": [
+    {"Target": "TheWanderer", "Favorability": 10},
+    {"Target": "ClanStonefist", "Favorability": 35},
+    {"Target": "Thrain", "Favorability": 30},
+    {"Target": "Bram", "Favorability": 25},
+    {"Target": "TheIronGuard", "Favorability": 20}
+  ],
+  "NPCLog": []
+}
+Kira: {
+  "Name": "Kira",
+  "NamePossessive": "Kira's",
+  "Species": "Human",
+  "HomeLocation": "PortFrost",
+  "CurrentLocation": "PortFrost",
+  "Faction": null,
+  "OwnedItems": {
+    "FishingRod": 1,
+    "GoldCoin": 10,
+    "Bread": 3
+  },
+  "Role": "Fisherman",
+  "Relations": [
+    {"Target": "TheWanderer", "Favorability": 15},
+    {"Target": "MerchantsGuild", "Favorability": 10},
+    {"Target": "Tessa", "Favorability": 15},
+    {"Target": "Percival", "Favorability": 10}
+  ],
+  "NPCLog": []
+}
+Magnus: {
+  "Name": "Magnus",
+  "NamePossessive": "Magnus'",
+  "Species": "Dwarf",
+  "HomeLocation": "Ironpeak",
+  "CurrentLocation": "Ironpeak",
+  "Faction": "ClanStonefist",
+  "OwnedItems": {
+    "SteelShield": 1,
+    "IronSword": 1,
+    "DwarvenAle": 4
+  },
+  "Role": "GuardCaptain",
+  "Relations": [
+    {"Target": "TheWanderer", "Favorability": 20},
+    {"Target": "ClanStonefist", "Favorability": 45},
+    {"Target": "Thrain", "Favorability": 35},
+    {"Target": "Roric", "Favorability": 30},
+    {"Target": "Gromm", "Favorability": -35}
+  ],
+  "NPCLog": []
+}
+Reyna: {
+  "Name": "Reyna",
+  "NamePossessive": "Reyna's",
+  "Species": "Human",
+  "HomeLocation": "Stonehaven",
+  "CurrentLocation": "Stonehaven",
+  "Faction": "TheIronGuard",
+  "OwnedItems": {
+    "IronDagger": 1,
+    "LeatherArmor": 1,
+    "Lockpick": 3
+  },
+  "Role": "Spy",
+  "Relations": [
+    {"Target": "TheWanderer", "Favorability": 10},
+    {"Target": "TheIronGuard", "Favorability": 35},
+    {"Target": "Borris", "Favorability": 30},
+    {"Target": "Valeria", "Favorability": 30},
+    {"Target": "Cyrus", "Favorability": -25}
+  ],
+  "NPCLog": []
+}
+Theron: {
+  "Name": "Theron",
+  "NamePossessive": "Theron's",
+  "Species": "Lizardfolk",
+  "HomeLocation": "CrimsonBadlands",
+  "CurrentLocation": "CrimsonBadlands",
+  "Faction": "CrimsonOutriders",
+  "OwnedItems": {
+    "IronSword": 1,
+    "TrollFat": 3,
+    "WolfPelt": 2
+  },
+  "Role": "Hunter",
+  "Relations": [
+    {"Target": "TheWanderer", "Favorability": -25},
+    {"Target": "CrimsonOutriders", "Favorability": 30},
+    {"Target": "Gromm", "Favorability": 25},
+    {"Target": "Kaelen", "Favorability": 25},
+    {"Target": "Eldrin", "Favorability": -20},
+    {"Target": "Isolde", "Favorability": -15}
+  ],
+  "NPCLog": []
+}
+Seraphina: {
+  "Name": "Seraphina",
+  "NamePossessive": "Seraphina's",
+  "Species": "Elf",
+  "HomeLocation": "Ravenwood",
+  "CurrentLocation": "Shadowmere",
+  "Faction": "CircleOfWhispers",
+  "OwnedItems": {
+    "MagesStaff": 1,
+    "ManaPotion": 5,
+    "AncientScroll": 2
+  },
+  "Role": "Wizard",
+  "Relations": [
+    {"Target": "TheWanderer", "Favorability": 15},
+    {"Target": "CircleOfWhispers", "Favorability": 30},
+    {"Target": "Eldrin", "Favorability": 20},
+    {"Target": "Cyrus", "Favorability": 20},
+    {"Target": "Valeria", "Favorability": -10}
+  ],
+  "NPCLog": []
+}
+Zephyr: {
+  "Name": "Zephyr",
+  "NamePossessive": "Zephyr's",
+  "Species": "Halfling",
+  "HomeLocation": "SunkissedFields",
+  "CurrentLocation": "SunkissedFields",
+  "Faction": null,
+  "OwnedItems": {
+    "Bread": 5,
+    "HealthPotion": 2,
+    "GoldCoin": 5
+  },
+  "Role": "Farmer",
+  "Relations": [
+    {"Target": "TheWanderer", "Favorability": 25},
+    {"Target": "Willow", "Favorability": 30},
+    {"Target": "Milo", "Favorability": 20},
+    {"Target": "Rosie", "Favorability": 25}
+  ],
+  "NPCLog": []
+}
+Corvus: {
+  "Name": "Corvus",
+  "NamePossessive": "Corvus'",
+  "Species": "Human",
+  "HomeLocation": "Shadowmere",
+  "CurrentLocation": "Shadowmere",
+  "Faction": "CircleOfWhispers",
+  "OwnedItems": {
+    "IronDagger": 1,
+    "Lockpick": 8,
+    "ThievesGuildMissive": 1
+  },
+  "Role": "Thief",
+  "Relations": [
+    {"Target": "TheWanderer", "Favorability": -5},
+    {"Target": "CircleOfWhispers", "Favorability": 40},
+    {"Target": "Nyx", "Favorability": 35},
+    {"Target": "Vex", "Favorability": 30},
+    {"Target": "Borris", "Favorability": -35},
+    {"Target": "Eldrin", "Favorability</t>
+  </si>
+  <si>
+    <t>test</t>
+  </si>
+  <si>
+    <t>data</t>
+  </si>
+  <si>
+    <t xml:space="preserve">## ENUM DATA
+{
+  "Types": {
+    "ItemTypes": ["Weapon", "Armor", "Potion", "Ingredient", "Key", "Artifact", "Currency", "Shield", "Scroll", "Tool"],
+    "QuestTypes": ["AttackThreateningEntities", "RecoverStolenItem", "GuardEntity", "AttackEnemy", "StealStuff", "KillEnemies"],
+    "EventTypes": ["Ambush", "Discovery", "Betrayal", "Alliance", "TradeRouteOpened", "ResourceDepleted", "Feast", "Plague", "RefugeeCrisis"],
+    "RelationshipLevels": {"Sworn Enemy": -50, "Enemy": -30, "Hated": -15, "Disliked": -5, "Neutral": 0, "Friendly": 5, "Friend": 15, "Ally": 30, "Sworn Ally": 50}
+  },
+  "Lists": {
+    "Species": ["Human", "Elf", "Dwarf", "Orc", "Halfling", "Lizardfolk", "Gnome", "Half-Elf", "Goblin", "Tiefling"],
+    "Roles": ["Innkeeper", "Blacksmith", "Merchant", "GuardCaptain", "Apothecary", "Thief", "Wizard", "Ranger", "Bard", "Priest", "Alchemist", "Farmer", "Mercenary", "Scholar", "Mayor", "Spy", "Hunter", "Fisherman", "Jeweler", "Scribe", "Stablemaster"],
+    "Locations": ["Eldrin Crossing", "Ironhold Keep", "Whispering Woods", "Sunken Harbor", "The Gilded Bazaar", "Ravenloft Cemetery", "Stormpeak Monastery", "Verdant Hollow", "The Ashen Scar", "Glimmerstone Caverns"],
+    "Factions": ["The Iron Circle", "Whisperwind Syndicate", "Order of the Verdant Flame", "The Rustwater Corsairs", "Gilded Consortium"],
+    "Enemies": ["Shadowmire Wolf", "Bone Wraith", "Cave Stalker", "Rustwater Raider", "Gloomspore Shambler", "Iron Circle Enforcer", "Verdant Protector", "Corsair Deckhand", "Syndicate Cutthroat", "Animated Armor", "Forest Lurker", "Ember Elemental", "Giant Spider", "Restless Soldier", "Cultist Acolyte", "Venomous Skitterer", "Bandit Marksman", "Corrupted Dryad", "Deep Gnawer", "Gargoyle Sentry"],
+    "Items": ["Iron Longsword", "Steel Dagger", "Elm Longbow", "Leather Jerkin", "Chainmail Hauberk", "Healing Salve", "Mana Draught", "Nightshade Petals", "Silver Dust", "Rusty Key", "Ancient Signet Ring", "Gold Crown", "Enchanted Vial", "Sturdy Shield", "Travelling Cloak", "Hunter's Trap", "Smoke Bomb", "Lockpicks", "Wolf Pelt", "Iron Ore", "Medical Kit", "Poison Vial", "Fire Bomb", "Strange Idol", "Star Map Fragment", "Unsent Letter"],
+    "NPCs": ["Elara Moonshadow", "Bram Ironfoot", "Grizzle Geargrinder", "Captain Valerius Stone", "Lysandra Vane", "Kaelen Swiftarrow", "Pippin Shortwick", "Sszarxis the Watcher", "Nissa Fizzlebang", "Brother Aldric", "Lyra Silvertongue", "Mira Thorne", "Drogan Shieldbiter", "Seraphina Goldleaf", "Old Man Hemlock", "Yorick the Gravedigger", "Tamsin Fleetwood", "Finnian Mossbrook", "Roderick Grimshaw", "Belladonna Shade", "Corporal Hayes", "Weylin Blackwater", "Garruk Steelwound", "Elowen Mistweaver", "Fenthwick Cobblepot", "Stitches Malone", "Marlowe Reed", "Greta Stonehearth", "Vex Holloway", "Torvin Coalbeard", "Anya Swift", "Silas the Tanner", "Petra Ironvein", "Quill Kettlewhistle", "Baelgor Thornwood", "Jasper Knackles", "Ser Varnholt", "Lilith Darkmoor", "Osric Cartwright", "Zephyr", "Boulder", "Glint", "Nyx", "Rattlebones", "Marrow", "Sable", "Whisper", "Orion Falkenrath", "Magnus Runehammer", "Caspian Voss", "The Warden"],
+    "Player": ["The Stranger"]
+  }
+}
+;
+### ITEM DATA
+Iron Longsword: { 
+  "Type": "Weapon", 
+  "Name": "Iron Longsword", 
+  "NameSingular": "Iron Longsword", 
+  "NamePlural": "Iron Longswords",
+  "NamePossessiveSingular": "Iron Longsword's",
+  "NamePossessivePlural": "Iron Longswords'",
+  "IndefiniteArticle": "an",
+  "IndefiniteArticleCaps": "An"
+}
+Steel Dagger: { 
+  "Type": "Weapon", 
+  "Name": "Steel Dagger", 
+  "NameSingular": "Steel Dagger", 
+  "NamePlural": "Steel Daggers",
+  "NamePossessiveSingular": "Steel Dagger's",
+  "NamePossessivePlural": "Steel Daggers'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+Elm Longbow: { 
+  "Type": "Weapon", 
+  "Name": "Elm Longbow", 
+  "NameSingular": "Elm Longbow", 
+  "NamePlural": "Elm Longbows",
+  "NamePossessiveSingular": "Elm Longbow's",
+  "NamePossessivePlural": "Elm Longbows'",
+  "IndefiniteArticle": "an",
+  "IndefiniteArticleCaps": "An"
+}
+Leather Jerkin: { 
+  "Type": "Armor", 
+  "Name": "Leather Jerkin", 
+  "NameSingular": "Leather Jerkin", 
+  "NamePlural": "Leather Jerkins",
+  "NamePossessiveSingular": "Leather Jerkin's",
+  "NamePossessivePlural": "Leather Jerkins'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+Chainmail Hauberk: { 
+  "Type": "Armor", 
+  "Name": "Chainmail Hauberk", 
+  "NameSingular": "Chainmail Hauberk", 
+  "NamePlural": "Chainmail Hauberks",
+  "NamePossessiveSingular": "Chainmail Hauberk's",
+  "NamePossessivePlural": "Chainmail Hauberks'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+Healing Salve: { 
+  "Type": "Potion", 
+  "Name": "Healing Salve", 
+  "NameSingular": "Healing Salve", 
+  "NamePlural": "Healing Salves",
+  "NamePossessiveSingular": "Healing Salve's",
+  "NamePossessivePlural": "Healing Salves'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+Mana Draught: { 
+  "Type": "Potion", 
+  "Name": "Mana Draught", 
+  "NameSingular": "Mana Draught", 
+  "NamePlural": "Mana Draughts",
+  "NamePossessiveSingular": "Mana Draught's",
+  "NamePossessivePlural": "Mana Draughts'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+Nightshade Petals: { 
+  "Type": "Ingredient", 
+  "Name": "Nightshade Petals", 
+  "NameSingular": "Nightshade Petal", 
+  "NamePlural": "Nightshade Petals",
+  "NamePossessiveSingular": "Nightshade Petal's",
+  "NamePossessivePlural": "Nightshade Petals'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+Silver Dust: { 
+  "Type": "Ingredient", 
+  "Name": "Silver Dust", 
+  "NameSingular": "Silver Dust", 
+  "NamePlural": "Silver Dust",
+  "NamePossessiveSingular": "Silver Dust's",
+  "NamePossessivePlural": "Silver Dust's",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+Rusty Key: { 
+  "Type": "Key", 
+  "Name": "Rusty Key", 
+  "NameSingular": "Rusty Key", 
+  "NamePlural": "Rusty Keys",
+  "NamePossessiveSingular": "Rusty Key's",
+  "NamePossessivePlural": "Rusty Keys'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+Ancient Signet Ring: { 
+  "Type": "Artifact", 
+  "Name": "Ancient Signet Ring", 
+  "NameSingular": "Ancient Signet Ring", 
+  "NamePlural": "Ancient Signet Rings",
+  "NamePossessiveSingular": "Ancient Signet Ring's",
+  "NamePossessivePlural": "Ancient Signet Rings'",
+  "IndefiniteArticle": "an",
+  "IndefiniteArticleCaps": "An"
+}
+Gold Crown: { 
+  "Type": "Currency", 
+  "Name": "Gold Crown", 
+  "NameSingular": "Gold Crown", 
+  "NamePlural": "Gold Crowns",
+  "NamePossessiveSingular": "Gold Crown's",
+  "NamePossessivePlural": "Gold Crowns'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+Enchanted Vial: { 
+  "Type": "Artifact", 
+  "Name": "Enchanted Vial", 
+  "NameSingular": "Enchanted Vial", 
+  "NamePlural": "Enchanted Vials",
+  "NamePossessiveSingular": "Enchanted Vial's",
+  "NamePossessivePlural": "Enchanted Vials'",
+  "IndefiniteArticle": "an",
+  "IndefiniteArticleCaps": "An"
+}
+Sturdy Shield: { 
+  "Type": "Shield", 
+  "Name": "Sturdy Shield", 
+  "NameSingular": "Sturdy Shield", 
+  "NamePlural": "Sturdy Shields",
+  "NamePossessiveSingular": "Sturdy Shield's",
+  "NamePossessivePlural": "Sturdy Shields'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+Travelling Cloak: { 
+  "Type": "Armor", 
+  "Name": "Travelling Cloak", 
+  "NameSingular": "Travelling Cloak", 
+  "NamePlural": "Travelling Cloaks",
+  "NamePossessiveSingular": "Travelling Cloak's",
+  "NamePossessivePlural": "Travelling Cloaks'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+Hunter's Trap: { 
+  "Type": "Tool", 
+  "Name": "Hunter's Trap", 
+  "NameSingular": "Hunter's Trap", 
+  "NamePlural": "Hunter's Traps",
+  "NamePossessiveSingular": "Hunter's Trap's",
+  "NamePossessivePlural": "Hunter's Traps'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+Smoke Bomb: { 
+  "Type": "Tool", 
+  "Name": "Smoke Bomb", 
+  "NameSingular": "Smoke Bomb", 
+  "NamePlural": "Smoke Bombs",
+  "NamePossessiveSingular": "Smoke Bomb's",
+  "NamePossessivePlural": "Smoke Bombs'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+Lockpicks: { 
+  "Type": "Tool", 
+  "Name": "Lockpicks", 
+  "NameSingular": "Lockpick", 
+  "NamePlural": "Lockpicks",
+  "NamePossessiveSingular": "Lockpick's",
+  "NamePossessivePlural": "Lockpicks'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+Wolf Pelt: { 
+  "Type": "Ingredient", 
+  "Name": "Wolf Pelt", 
+  "NameSingular": "Wolf Pelt", 
+  "NamePlural": "Wolf Pelts",
+  "NamePossessiveSingular": "Wolf Pelt's",
+  "NamePossessivePlural": "Wolf Pelts'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+Iron Ore: { 
+  "Type": "Ingredient", 
+  "Name": "Iron Ore", 
+  "NameSingular": "Iron Ore", 
+  "NamePlural": "Iron Ore",
+  "NamePossessiveSingular": "Iron Ore's",
+  "NamePossessivePlural": "Iron Ore's",
+  "IndefiniteArticle": "an",
+  "IndefiniteArticleCaps": "An"
+}
+Medical Kit: { 
+  "Type": "Tool", 
+  "Name": "Medical Kit", 
+  "NameSingular": "Medical Kit", 
+  "NamePlural": "Medical Kits",
+  "NamePossessiveSingular": "Medical Kit's",
+  "NamePossessivePlural": "Medical Kits'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+Poison Vial: { 
+  "Type": "Potion", 
+  "Name": "Poison Vial", 
+  "NameSingular": "Poison Vial", 
+  "NamePlural": "Poison Vials",
+  "NamePossessiveSingular": "Poison Vial's",
+  "NamePossessivePlural": "Poison Vials'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+Fire Bomb: { 
+  "Type": "Tool", 
+  "Name": "Fire Bomb", 
+  "NameSingular": "Fire Bomb", 
+  "NamePlural": "Fire Bombs",
+  "NamePossessiveSingular": "Fire Bomb's",
+  "NamePossessivePlural": "Fire Bombs'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+Strange Idol: { 
+  "Type": "Artifact", 
+  "Name": "Strange Idol", 
+  "NameSingular": "Strange Idol", 
+  "NamePlural": "Strange Idols",
+  "NamePossessiveSingular": "Strange Idol's",
+  "NamePossessivePlural": "Strange Idols'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+Star Map Fragment: { 
+  "Type": "Artifact", 
+  "Name": "Star Map Fragment", 
+  "NameSingular": "Star Map Fragment", 
+  "NamePlural": "Star Map Fragments",
+  "NamePossessiveSingular": "Star Map Fragment's",
+  "NamePossessivePlural": "Star Map Fragments'",
+  "IndefiniteArticle": "a",
+  "IndefiniteArticleCaps": "A"
+}
+Unsent Letter: { 
+  "Type": "Artifact", 
+  "Name": "Unsent Letter", 
+  "NameSingular": "Unsent Letter", 
+  "NamePlural": "Unsent Letters",
+  "NamePossessiveSingular": "Unsent Letter's",
+  "NamePossessivePlural": "Unsent Letters'",
+  "IndefiniteArticle": "an",
+  "IndefiniteArticleCaps": "An"
+}
+;
+## GAME STATE DATA
+### FACTION DATA
+The Iron Circle: {
+  "Name": "The Iron Circle", 
+  "NameDefinitive": "the Iron Circle",
+  "NameDefinitiveCaps": "The Iron Circle",
+  "NamePossessive": "The Iron Circle's",
+  "NameDefinitivePossessive": "the Iron Circle's",
+  "NameDefinitivePossessiveCaps": "The Iron Circle's",
+  "DefaultLocation": "Ironhold Keep",
+  "Relations": [
+    {"Target": "The Stranger", "Favorability": 15},
+    {"Target": "Whisperwind Syndicate", "Favorability": -30},
+    {"Target": "Order of the Verdant Flame", "Favorability": 5},
+    {"Target": "The Rustwater Corsairs", "Favorability": -15},
+    {"Target": "Gilded Consortium", "Favorability": 30}
+  ],
+  "Members": ["Bram Ironfoot", "Captain Valerius Stone", "Drogan Shieldbiter", "Corporal Hayes", "Garruk Steelwound", "Petra Ironvein", "Ser Varnholt", "Magnus Runehammer"],
+  "Treasury": {
+    "Iron Longsword": 12,
+    "Chainmail Hauberk": 8,
+    "Sturdy Shield": 15,
+    "Gold Crown": 2500,
+    "Iron Ore": 45
+  },
+  "FactionLog": []
+}
+Whisperwind Syndicate: {
+  "Name": "Whisperwind Syndicate", 
+  "NameDefinitive": "the Whisperwind Syndicate",
+  "NameDefinitiveCaps": "The Whisperwind Syndicate",
+  "NamePossessive": "Whisperwind Syndicate's",
+  "NameDefinitivePossessive": "the Whisperwind Syndicate's",
+  "NameDefinitivePossessiveCaps": "The Whisperwind Syndicate's",
+  "DefaultLocation": "The Gilded Bazaar",
+  "Relations": [
+    {"Target": "The Stranger", "Favorability": 5},
+    {"Target": "The Iron Circle", "Favorability": -30},
+    {"Target": "Order of the Verdant Flame", "Favorability": -15},
+    {"Target": "The Rustwater Corsairs", "Favorability": 15},
+    {"Target": "Gilded Consortium", "Favorability": -5}
+  ],
+  "Members": ["Lysandra Vane", "Lyra Silvertongue", "Belladonna Shade", "Weylin Blackwater", "Vex Holloway", "Jasper Knackles", "Sable", "Whisper", "Caspian Voss"],
+  "Treasury": {
+    "Steel Dagger": 20,
+    "Lockpicks": 30,
+    "Smoke Bomb": 45,
+    "Poison Vial": 18,
+    "Gold Crown": 5800
+  },
+  "FactionLog": []
+}
+Order of the Verdant Flame: {
+  "Name": "Order of the Verdant Flame", 
+  "NameDefinitive": "the Order of the Verdant Flame",
+  "NameDefinitiveCaps": "The Order of the Verdant Flame",
+  "NamePossessive": "Order of the Verdant Flame's",
+  "NameDefinitivePossessive": "the Order of the Verdant Flame's",
+  "NameDefinitivePossessiveCaps": "The Order of the Verdant Flame's",
+  "DefaultLocation": "Verdant Hollow",
+  "Relations": [
+    {"Target": "The Stranger", "Favorability": 30},
+    {"Target": "The Iron Circle", "Favorability": 5},
+    {"Target": "Whisperwind Syndicate", "Favorability": -15},
+    {"Target": "The Rustwater Corsairs", "Favorability": -50},
+    {"Target": "Gilded Consortium", "Favorability": 0}
+  ],
+  "Members": ["Kaelen Swiftarrow", "Mira Thorne", "Seraphina Goldleaf", "Finnian Mossbrook", "Elowen Mistweaver", "Anya Swift", "Baelgor Thornwood", "Orion Falkenrath"],
+  "Treasury": {
+    "Elm Longbow": 15,
+    "Leather Jerkin": 10,
+    "Healing Salve": 40,
+    "Mana Draught": 25,
+    "Nightshade Petals": 60
+  },
+  "FactionLog": []
+}
+The Rustwater Corsairs: {
+  "Name": "The Rustwater Corsairs", 
+  "NameDefinitive": "the Rustwater Corsairs",
+  "NameDefinitiveCaps": "The Rustwater Corsairs",
+  "NamePossessive": "The Rustwater Corsairs'",
+  "NameDefinitivePossessive": "the Rustwater Corsairs'",
+  "NameDefinitivePossessiveCaps": "The Rustwater Corsairs'",
+  "DefaultLocation": "Sunken Harbor",
+  "Relations": [
+    {"Target": "The Stranger", "Favorability": -15},
+    {"Target": "The Iron Circle", "Favorability": -15},
+    {"Target": "Whisperwind Syndicate", "Favorability": 15},
+    {"Target": "Order of the Verdant Flame", "Favorability": -50},
+    {"Target": "Gilded Consortium", "Favorability": -5}
+  ],
+  "Members": ["Captain Valerius Stone", "Tamsin Fleetwood", "Roderick Grimshaw", "Marlowe Reed", "Greta Stonehearth", "Lilith Darkmoor", "Boulder", "Nyx"],
+  "Treasury": {
+    "Steel Dagger": 30,
+    "Gold Crown": 12000,
+    "Unsent Letter": 5,
+    "Star Map Fragment": 2,
+    "Smoke Bomb": 10
+  },
+  "FactionLog": []
+}
+Gilded Consortium: {
+  "Name": "Gilded Consortium", 
+  "NameDefinitive": "the Gilded Consortium",
+  "NameDefinitiveCaps": "The Gilded Consortium",
+  "NamePossessive": "Gilded Consortium's",
+  "NameDefinitivePossessive": "the Gilded Consortium's",
+  "NameDefinitivePossessiveCaps": "The Gilded Consortium's",
+  "DefaultLocation": "Eldrin Crossing",
+  "Relations": [
+    {"Target": "The Stranger", "Favorability": 5},
+    {"Target": "The Iron Circle", "Favorability": 30},
+    {"Target": "Whisperwind Syndicate", "Favorability": -5},
+    {"Target": "Order of the Verdant Flame", "Favorability": 0},
+    {"Target": "The Rustwater Corsairs", "Favorability": -5}
+  ],
+  "Members": ["Grizzle Geargrinder", "Pippin Shortwick", "Nissa Fizzlebang", "Fenthwick Cobblepot", "Stitches Malone", "Torvin Coalbeard", "Quill Kettlewhistle", "Osric Cartwright", "Glint"],
+  "Treasury": {
+    "Gold Crown": 15000,
+    "Silver Dust": 80,
+    "Enchanted Vial": 5,
+    "Ancient Signet Ring": 2,
+    "Travelling Cloak": 10
+  },
+  "FactionLog": []
+}
+;
+### NPC DATA
+Elara Moonshadow: {
+  "Name": "Elara Moonshadow",
+  "NamePossessive": "Elara Moonshadow's",
+  "Species": "Elf",
+  "HomeLocation": "Whispering Woods",
+  "CurrentLocation": "Eldrin Crossing",
+  "Faction": null,
+  "OwnedItems": {
+    "Elm Longbow": 1,
+    "Mana Draught": 3,
+    "Star Map Fragment": 1
+  },
+  "Role": "Ranger",
+  "Relations": [
+    {"Target": "The Stranger", "Favorability": 15},
+    {"Target": "Order of the Verdant Flame", "Favorability": 30},
+    {"Target": "The Rustwater Corsairs", "Favorability": -30},
+    {"Target": "Kaelen Swiftarrow", "Favorability": 25},
+    {"Target": "Roderick Grimshaw", "Favorability": -40},
+    {"Target": "Mira Thorne", "Favorability": 10}
+  ],
+  "NPCLog": []
+}
+Bram Ironfoot: {
+  "Name": "Bram Ironfoot",
+  "NamePossessive": "Bram Ironfoot's",
+  "Species": "Dwarf",
+  "HomeLocation": "Ironhold Keep",
+  "CurrentLocation": "Ironhold Keep",
+  "Faction": "The Iron Circle",
+  "OwnedItems": {
+    "Chainmail Hauberk": 1,
+    "Iron Longsword": 1,
+    "Sturdy Shield": 1
+  },
+  "Role": "GuardCaptain",
+  "Relations": [
+    {"Target": "The Stranger", "Favorability": 15},
+    {"Target": "The Iron Circle", "Favorability": 50},
+    {"Target": "Whisperwind Syndicate", "Favorability": -15},
+    {"Target": "Captain Valerius Stone", "Favorability": 20},
+    {"Target": "Lysandra Vane", "Favorability": -10},
+    {"Target": "Drogan Shieldbiter", "Favorability": 30}
+  ],
+  "NPCLog": []
+}
+Grizzle Geargrinder: {
+  "Name": "Grizzle Geargrinder",
+  "NamePossessive": "Grizzle Geargrinder's",
+  "Species": "Gnome",
+  "HomeLocation": "Eldrin Crossing",
+  "CurrentLocation": "Eldrin Crossing",
+  "Faction": "Gilded Consortium",
+  "OwnedItems": {
+    "Lockpicks": 1,
+    "Enchanted Vial": 1,
+    "Silver Dust": 5
+  },
+  "Role": "Blacksmith",
+  "Relations": [
+    {"Target": "The Stranger", "Favorability": 5},
+    {"Target": "Gilded Consortium", "Favorability": 30},
+    {"Target": "The Iron Circle", "Favorability": 15},
+    {"Target": "Pippin Shortwick", "Favorability": 20},
+    {"Target": "Torvin Coalbeard", "Favorability": 10}
+  ],
+  "NPCLog": []
+}
+Captain Valerius Stone: {
+  "Name": "Captain Valerius Stone",
+  "NamePossessive": "Captain Valerius Stone's",
+  "Species": "Human",
+  "HomeLocation": "Ironhold Keep",
+  "CurrentLocation": "Sunken Harbor",
+  "Faction": "The Rustwater Corsairs",
+  "OwnedItems": {
+    "Steel Dagger": 1,
+    "Star Map Fragment": 1,
+    "Gold Crown": 150
+  },
+  "Role": "Mercenary",
+  "Relations": [
+    {"Target": "The Stranger", "Favorability": -15},
+    {"Target": "The Rustwater Corsairs", "Favorability": 30},
+    {"Target": "Order of the Verdant Flame", "Favorability": -40},
+    {"Target": "Bram Ironfoot", "Favorability": 20},
+    {"Target": "Kaelen Swiftarrow", "Favorability": -25}
+  ],
+  "NPCLog": []
+}
+Lysandra Vane: {
+  "Name": "Lysandra Vane",
+  "NamePossessive": "Lysandra Vane's",
+  "Species": "Half-Elf",
+  "HomeLocation": "The Gilded Bazaar",
+  "CurrentLocation": "The Gilded Bazaar",
+  "Faction": "Whisperwind Syndicate",
+  "OwnedItems": {
+    "Steel Dagger": 2,
+    "Poison Vial": 3,
+    "Smoke Bomb": 5
+  },
+  "Role": "Spy",
+  "Relations": [
+    {"Target": "The Stranger", "Favorability": 5},
+    {"Target": "Whisperwind Syndicate", "Favorability": 30},
+    {"Target": "The Iron Circle", "Favorability": -30},
+    {"Target": "Belladonna Shade", "Favorability": 15},
+    {"Target": "Bram Ironfoot", "Favorability": -20}
+  ],
+  "NPCLog": []
+}
+Kaelen Swiftarrow: {
+  "Name": "Kaelen Swiftarrow",
+  "NamePossessive": "Kaelen Swiftarrow's",
+  "Species": "Elf",
+  "HomeLocation": "Verdant Hollow",
+  "CurrentLocation": "Verdant Hollow",
+  "Faction": "Order of the Verdant Flame",
+  "OwnedItems": {
+    "Elm Longbow": 1,
+    "Leather Jerkin": 1,
+    "Healing Salve": 2
+  },
+  "Role": "Ranger",
+  "Relations": [
+    {"Target": "The Stranger", "Favorability": 25},
+    {"Target": "Order of the Verdant Flame", "Favorability": 50},
+    {"Target": "The Rustwater Corsairs", "Favorability": -50},
+    {"Target": "Elara Moonshadow", "Favorability": 25},
+    {"Target": "Captain Valerius Stone", "Favorability": -50}
+  ],
+  "NPCLog": []
+}
+Pippin Shortwick: {
+  "Name": "Pippin Shortwick",
+  "NamePossessive": "Pippin Shortwick's",
+  "Species": "Halfling",
+  "HomeLocation": "Eldrin Crossing",
+  "CurrentLocation": "Eldrin Crossing",
+  "Faction": "Gilded Consortium",
+  "OwnedItems": {
+    "Travelling Cloak": 1,
+    "Gold Crown": 50,
+    "Lockpicks": 1
+  },
+  "Role": "Merchant",
+  "Relations": [
+    {"Target": "The Stranger", "Favorability": 10},
+    {"Target": "Gilded Consortium", "Favorability": 15},
+    {"Target": "Whisperwind Syndicate", "Favorability": -5},
+    {"Target": "Nissa Fizzlebang", "Favorability": 20},
+    {"Target": "Lyra Silvertongue", "Favorability": -10}
+  ],
+  "NPCLog": []
+}
+Sszarxis the Watcher: {
+  "Name": "Sszarxis the Watcher",
+  "NamePossessive": "Sszarxis the Watcher's",
+  "Species": "Lizardfolk",
+  "HomeLocation": "Sunken Harbor",
+  "CurrentLocation": "Sunken Harbor",
+  "Faction": null,
+  "OwnedItems": {
+    "Strange Idol": 1,
+    "Wolf Pelt": 3,
+    "Nightshade Petals": 10
+  },
+  "Role": "Hunter",
+  "Relations": [
+    {"Target": "The Stranger", "Favorability": 0},
+    {"Target": "The Rustwater Corsairs", "Favorability": -5},
+    {"Target": "Order of the Verdant Flame", "Favorability": 15},
+    {"Target": "Marlowe Reed", "Favorability": -15}
+  ],
+  "NPCLog": []
+}
+Nissa Fizzlebang: {
+  "Name": "Nissa Fizzlebang",
+  "NamePossessive": "Nissa Fizzlebang's",
+  "Species": "Gnome",
+  "HomeLocation": "Eldrin Crossing",
+  "CurrentLocation": "Glimmerstone Caverns",
+  "Faction": "Gilded Consortium",
+  "OwnedItems": {
+    "Enchanted Vial": 2,
+    "Silver Dust": 10,
+    "Mana Draught": 3
+  },
+  "Role": "Alchemist",
+  "Relations": [
+    {"Target": "The Stranger", "Favorability": 5},
+    {"Target": "Gilded Consortium", "Favorability": 15},
+    {"Target": "Pippin Shortwick", "Favorability": 20},
+    {"Target": "Fenthwick Cobblepot", "Favorability": -5}
+  ],
+  "NPCLog": []
+}
+Brother Aldric: {
+  "Name": "Brother Aldric",
+  "NamePossessive": "Brother Aldric's",
+  "Species": "Human",
+  "HomeLocation": "Stormpeak Monastery",
+  "CurrentLocation": "Stormpeak Monastery",
+  "Faction": null,
+  "OwnedItems": {
+    "Medical Kit": 1,
+    "Healing Salve": 5,
+    "Ancient Signet Ring": 1
+  },
+  "Role": "Priest",
+  "Relations": [
+    {"Target": "The Stranger", "Favorability": 20},
+    {"Target": "Order of the Verdant Flame", "Favorability": 30},
+    {"Target": "The Rustwater Corsairs", "Favorability": -15},
+    {"Target": "Ser Varnholt", "Favorability": 10},
+    {"Target": "Lilith Darkmoor", "Favorability": -25}
+  ],
+  "NPCLog": []
+}
+Lyra Silvertongue: {
+  "Name": "Lyra Silvertongue",
+  "NamePossessive": "Lyra Silvertongue's",
+  "Species": "Tiefling",
+  "HomeLocation": "The Gilded Bazaar",
+  "CurrentLocation": "Eldrin Crossing",
+  "Faction": "Whisperwind Syndicate",
+  "OwnedItems": {
+    "Steel Dagger": 1,
+    "Poison Vial": 2,
+    "Unsent Letter": 1
+  },
+  "Role": "Bard",
+  "Relations": [
+    {"Target": "The Stranger", "Favorability": -5},
+    {"Target": "Whisperwind Syndicate", "Favorability": 15},
+    {"Target": "The Iron Circle", "Favorability": -15},
+    {"Target": "Belladonna Shade", "Favorability": -10},
+    {"Target": "Pippin Shortwick", "Favorability": -10}
+  ],
+  "NPCLog": []
+}
+Mira Thorne: {
+  "Name": "Mira Thorne",
+  "NamePossessive": "Mira Thorne's",
+  "Species": "Half-Elf",
+  "HomeLocation": "Verdant Hollow",
+  "CurrentLocation": "Whispering Woods",
+  "Faction": "Order of the Verdant Flame",
+  "OwnedItems": {
+    "Mana Draught": 5,
+    "Nightshade Petals": 8,
+    "Healing Salve": 2
+  },
+  "Role": "Apothecary",
+  "Relations": [
+    {"Target": "The Stranger", "Favorability": 30},
+    {"Target": "Order of the Verdant Flame", "Favorability": 30},
+    {"Target": "Elara Moonshadow", "Favorability": 10},
+    {"Target": "Sszarxis the Watcher", "Favorability": 5}
+  ],
+  "NPCLog": []
+}
+Drogan Shieldbiter: {
+  "Name": "Drogan Shieldbiter",
+  "NamePossessive": "Drogan Shieldbiter's",
+  "Species": "Dwarf",
+  "HomeLocation": "Ironhold Keep",
+  "CurrentLocation": "Ironhold Keep",
+  "Faction": "The Iron Circle",
+  "OwnedItems": {
+    "Iron Longsword": 1,
+    "Sturdy Shield": 1,
+    "Iron Ore": 5
+  },
+  "Role": "Blacksmith",
+  "Relations": [
+    {"Target": "The Stranger", "Favorability": 10},
+    {"Target": "The Iron Circle", "Favorability": 50},
+    {"Target": "Gilded Consortium", "Favorability": 5},
+    {"Target": "Bram Ironfoot", "Favorability": 30},
+    {"Target": "Grizzle Geargrinder", "Favorability": 15}
+  ],
+  "NPCLog": []
+}
+Seraphina Goldleaf: {
+  "Name": "Seraphina Goldleaf",
+  "NamePossessive": "Seraphina Goldleaf's",
+  "Species": "Elf",
+  "HomeLocation": "Verdant Hollow",
+  "CurrentLocation": "Verdant Hollow",
+  "Faction": "Order of the Verdant Flame",
+  "OwnedItems": {
+    "Enchanted Vial": 1,
+    "Mana Draught": 4,
+    "Star Map Fragment": 1
+  },
+  "Role": "Wizard",
+  "Relations": [
+    {"Target": "The Stranger", "Favorability": 35},
+    {"Target": "Order of the Verdant Flame", "Favorability": 40},
+    {"Target": "The Rustwater Corsairs", "Favorability": -50},
+    {"Target": "Kaelen Swiftarrow", "Favorability": 15},
+    {"Target": "Elara Moonshadow", "Favorability": 20}
+  ],
+  "NPCLog": []
+}
+Old Man Hemlock: {
+  "Name": "Old Man Hemlock",
+  "NamePossessive": "Old Man Hemlock's",
+  "Species": "Human",
+  "HomeLocation": "Ravenloft Cemetery",
+  "CurrentLocation": "Ravenloft Cemetery",
+  "Faction": null,
+  "OwnedItems": {
+    "Rusty Key": 1,
+    "Wolf Pelt": 2,
+    "Strange Idol": 1
+  },
+  "Role": "Priest",
+  "Relations": [
+    {"Target": "The Stranger", "Favorability": -5},
+    {"Target": "Yorick the Gravedigger", "Favorability": 15},
+    {"Target": "Belladonna Shade", "Favorability": -20}
+  ],
+  "NPCLog": []
+}
+Yorick the Gravedigger: {
+  "Name": "Yorick the Gravedigger",
+  "NamePossessive": "Yorick the Gravedigger's",
+  "Species": "Human",
+  "HomeLocation": "Ravenloft Cemetery",
+  "CurrentLocation": "Ravenloft Cemetery",
+  "Faction": null,
+  "OwnedItems": {
+    "Iron Longsword": 1,
+    "Medical Kit": 1,
+    "Wolf Pelt": 1
+  },
+  "Role": "Mercenary",
+  "Relations": [
+    {"Target": "The Stranger", "Favorability": 0},
+    {"Target": "Old Man Hemlock", "Favorability": 15},
+    {"Target": "The Rustwater Corsairs", "Favorability": -15}
+  ],
+  "NPCLog": []
+}
+Tamsin Fleetwood: {
+  "Name": "Tamsin Fleetwood",
+  "NamePossessive": "Tamsin Fleetwood's",
+  "Species": "Human",
+  "HomeLocation": "Sunken Harbor",
+  "CurrentLocation": "Sunken Harbor",
+  "Faction": "The Rustwater Corsairs",
+  "OwnedItems": {
+    "Steel Dagger": 1,
+    "Smoke Bomb": 2,
+    "Gold Crown": 80
+  },
+  "Role": "Fisherman",
+  "Relations": [
+    {"Target": "The Stranger", "Favorability": -10},
+    {"Target": "The Rustwater Corsairs", "Favorability": 15},
+    {"Target": "Order of the Verdant Flame", "Favorability": -30},
+    {"Target": "Marlowe Reed", "Favorability": 10}
+  ],
+  "NPCLog": []
+}
+Finnian Mossbrook: {
+  "Name": "Finnian Mossbrook",
+  "NamePossessive": "Finnian Mossbrook's",
+  "Species": "Halfling",
+  "HomeLocation": "Verdant Hollow",
+  "CurrentLocation": "Whispering Woods",
+  "Faction": "Order of the Verdant Flame",
+  "OwnedItems": {
+    "Healing Salve": 3,
+    "Nightshade Petals": 5,
+    "Hunter's Trap": 2
+  },
+  "Role": "Hunter",
+  "Relations": [
+    {"Target": "The Stranger", "Favorability": 15},
+    {"Target": "Order of the Verdant Flame", "Favorability": 30},
+    {"Target": "Sszarxis the Watcher", "Favorability": 5},
+    {"Target": "Mira Thorne", "Favorability": 20}
+  ],
+  "NPCLog": []
+}
+Roderick Grimshaw: {
+  "Name": "Roderick Grimshaw",
+  "NamePossessive": "Roderick Grimshaw's",
+  "Species": "Half-Elf",
+  "HomeLocation": "Sunken Harbor",
+  "CurrentLocation": "The Ashen Scar",
+  "Faction": "The Rustwater Corsairs",
+  "OwnedItems": {
+    "Steel Dagger": 1,
+    "Poison Vial": 2,
+    "Fire Bomb": 3
+  },
+  "Role": "Thief",
+  "Relations": [
+    {"Target": "The Stranger", "Favorability": -50},
+    {"Target": "The Rustwater Corsairs", "Favorability": 30},
+    {"Target": "Order of the Verdant Flame", "Favorability": -50},
+    {"Target": "Elara Moonshadow", "Favorability": -40},
+    {"Target": "Lysandra Vane", "Favorability": 10}
+  ],
+  "NPCLog": []
+}
+Belladonna Shade: {
+  "Name": "Belladonna Shade",
+  "NamePossessive": "Belladonna Shade's",
+  "Species": "Tiefling",
+  "HomeLocation": "The Gilded Bazaar",
+  "CurrentLocation": "The Gilded Bazaar",
+  "Faction": "Whisperwind Syndicate",
+  "OwnedItems": {
+    "Poison Vial": 5,
+    "Nightshade Petals": 15,
+    "Lockpicks": 1
+  },
+  "Role": "Alchemist",
+  "Relations": [
+    {"Target": "The Stranger", "Favorability": -15},
+    {"Target": "Whisperwind Syndicate", "Favorability": 30},
+    {"Target": "The Iron Circle", "Favorability": -30},
+    {"Target": "Lyra Silvertongue", "Favorability": -10},
+    {"Target": "Lysandra Vane", "Favorability": 15}
+  ],
+  "NPCLog": []
+}
+Corporal Hayes: {
+  "Name": "Corporal Hayes",
+  "NamePossessive": "Corporal Hayes'",
+  "Species": "Human",
+  "HomeLocation": "Ironhold Keep",
+  "CurrentLocation": "Ironhold Keep",
+  "Faction": "The Iron Circle",
+  "OwnedItems": {
+    "Chainmail Hauberk": 1,
+    "Iron Longsword": 1,
+    "Medical Kit": 1
+  },
+  "Role": "GuardCaptain",
+  "Relations": [
+    {"Target": "The Stranger", "Favorability": 15},
+    {"Target": "The Iron Circle", "Favorability": 40},
+    {"Target": "Bram Ironfoot", "Favorability": 25},
+    {"Target": "Drogan Shieldbiter", "Favorability": 20}
+  ],
+  "NPCLog": []
+}
+Weylin Blackwater: {
+  "Name": "Weylin Blackwater",
+  "NamePossessive": "Weylin Blackwater's",
+  "Species": "Human",
+  "HomeLocation": "Sunken Harbor",
+  "CurrentLocation": "The Gilded Bazaar",
+  "Faction": "Whisperwind Syndicate",
+  "OwnedItems": {
+    "Smoke Bomb": 3,
+    "Steel Dagger": 1,
+    "Unsent Letter": 1
+  },
+  "Role": "Spy",
+  "Relations": [
+    {"Target": "The Stranger", "Favorability": -5},
+    {"Target": "Whisperwind Syndicate", "Favorability": 15},
+    {"Target": "The Rustwater Corsairs", "Favorability": 5},
+    {"Target": "Lysandra Vane", "Favorability": 10}
+  ],
+  "NPCLog": []
+}
+Garruk Steelwound: {
+  "Name": "Garruk Steelwound",
+  "NamePossessive": "Garruk Steelwound's",
+  "Species": "Orc",
+  "HomeLocation": "Ironhold Keep",
+  "CurrentLocation": "Ironhold Keep",
+  "Faction": "The Iron Circle",
+  "OwnedItems": {
+    "Iron Longsword": 1,
+    "Sturdy Shield": 1,
+    "Wolf Pelt": 2
+  },
+  "Role": "Mercenary",
+  "Relations": [
+    {"Target": "The Stranger", "Favorability": 20},
+    {"Target": "The Iron Circle", "Favorability": 30},
+    {"Target": "Order of the Verdant Flame", "Favorability": -5},
+    {"Target": "Bram Ironfoot", "Favorability": 15}
+  ],
+  "NPCLog": []
+}
+Elowen Mistweaver: {
+  "Name": "Elowen Mistweaver",
+  "NamePossessive": "Elowen Mistweaver's",
+  "Species": "Elf",
+  "HomeLocation": "Verdant Hollow",
+  "CurrentLocation": "Glimmerstone Caverns",
+  "Faction": "Order of the Verdant Flame",
+  "OwnedItems": {
+    "Mana Draught": 4,
+    "Enchanted Vial": 1,
+    "Silver Dust": 10
+  },
+  "Role": "Wizard",
+  "Relations": [
+    {"Target": "The Stranger", "Favorability": 25},
+    {"Target": "Order of the Verdant Flame", "Favorability": 40},
+    {"Target": "Nissa Fizzlebang", "Favorability": 15}
+  ],
+  "NPCLog": []
+}
+Fenthwick Cobblepot: {
+  "Name": "Fenthwick Cobblepot",
+  "NamePossessive": "Fenthwick Cobblepot's",
+  "Species": "Gnome",
+  "HomeLocation": "Eldrin Crossing",
+  "CurrentLocation": "Eldrin Crossing",
+  "Faction": "Gilded Consortium",
+  "OwnedItems": {
+    "Lockpicks": 1,
+    "Travelling Cloak": 1,
+    "Gold Crown": 200
+  },
+  "Role": "Merchant",
+  "Relations": [
+    {"Target": "The Stranger", "Favorability": 5},
+    {"Target": "Gilded Consortium", "Favorability": 20},
+    {"Target": "Pippin Shortwick", "Favorability": 15},
+    {"Target": "Nissa Fizzlebang", "Favorability": -5}
+  ],
+  "NPCLog": []
+}
+Stitches Malone: {
+  "Name": "Stitches Malone",
+  "NamePossessive": "Stitches Malone's",
+  "Species": "Human",
+  "HomeLocation": "Eldrin Crossing",
+  "CurrentLocation": "Eldrin Crossing",
+  "Faction": "Gilded Consortium",
+  "OwnedItems": {
+    "Medical Kit": 2,
+    "Healing Salve": 5,
+    "Silver Dust": 3
+  },
+  "Role": "Apothecary",
+  "Relations": [
+    {"Target": "The Stranger", "Favorability": 10},
+    {"Target": "Gilded Consortium", "Favorability": 15},
+    {"Target": "Mira Thorne", "Favorability": 5}
+  ],
+  "NPCLog": []
+}
+Marlowe Reed: {
+  "Name": "Marlowe Reed",
+  "NamePossessive": "Marlowe Reed's",
+  "Species": "Halfling",
+  "HomeLocation": "Sunken Harbor",
+  "CurrentLocation": "Sunken Harbor",
+  "Faction": "The Rustwater Corsairs",
+  "OwnedItems": {
+    "Smoke Bomb": 2,
+    "Steel Dagger": 1,
+    "Gold Crown": 120
+  },
+  "Role": "Thief",
+  "Relations": [
+    {"Target": "The Stranger", "Favorability": -10},
+    {"Target": "The Rustwater Corsairs", "Favorability": 15},
+    {"Target": "Tamsin Fleetwood", "Favorability": 10},
+    {"Target": "Sszarxis the Watcher", "Favorability": -15}
+  ],
+  "NPCLog": </t>
   </si>
 </sst>
 </file>
@@ -18686,6 +20738,7 @@
   <cols>
     <col min="1" max="1" width="11.5546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="24.21875" customWidth="1"/>
+    <col min="5" max="5" width="22.109375" customWidth="1"/>
     <col min="8" max="8" width="18.88671875" customWidth="1"/>
   </cols>
   <sheetData>
@@ -18696,6 +20749,12 @@
       <c r="B1" t="s">
         <v>1</v>
       </c>
+      <c r="D1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E1" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="2" spans="1:8" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
@@ -18703,6 +20762,12 @@
       </c>
       <c r="B2" s="3" t="s">
         <v>11</v>
+      </c>
+      <c r="D2" t="s">
+        <v>43</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>44</v>
       </c>
       <c r="H2" s="3"/>
     </row>
@@ -18840,7 +20905,7 @@
         <v>26</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -18848,14 +20913,16 @@
         <v>28</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B21" s="3"/>
+      <c r="B21" s="3" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="22" spans="1:2" ht="13.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
@@ -18880,5 +20947,6 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>